<commit_message>
Add MN-2007 alignment bridge — the current teaching framework
MN-2007 is the framework the department currently teaches from.
Built targeted bridge: CPM lesson → MN-2022 code → topic cluster → MN-2007 codes.
Also uses HS correlations sheet's direct MN-2022 ↔ MN-2007 column.

Results:
- MN-2007 Grade 6: 18/18 covered (0 gaps)
- MN-2007 Grade 7: 18/18 covered (0 gaps)
- MN-2007 Grade 8: 16/16 covered (0 gaps)
- CC1 now shows MN-2007 alignments (e.g., 1.1.2 → 6.3.1.1 Area & Geometry)
- All spreadsheets rebuilt with MN-2007 data
- 2,616 total alignments

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/export/alignment_report.xlsx
+++ b/export/alignment_report.xlsx
@@ -688,9 +688,9 @@
           <t>29/292</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>0/65</t>
+      <c r="E8" s="6" t="inlineStr">
+        <is>
+          <t>18/65</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -705,7 +705,7 @@
         <v>263</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>65</v>
+        <v>47</v>
       </c>
       <c r="J8" s="5" t="n">
         <v>360</v>
@@ -730,9 +730,9 @@
           <t>68/292</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>0/65</t>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>18/65</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -747,7 +747,7 @@
         <v>224</v>
       </c>
       <c r="I9" s="5" t="n">
-        <v>65</v>
+        <v>47</v>
       </c>
       <c r="J9" s="5" t="n">
         <v>360</v>
@@ -772,9 +772,9 @@
           <t>59/292</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>0/65</t>
+      <c r="E10" s="6" t="inlineStr">
+        <is>
+          <t>16/65</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -789,7 +789,7 @@
         <v>233</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>65</v>
+        <v>49</v>
       </c>
       <c r="J10" s="5" t="n">
         <v>360</v>
@@ -809,9 +809,9 @@
           <t>35/373</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>0/292</t>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>28/292</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -828,7 +828,7 @@
         <v>338</v>
       </c>
       <c r="H11" s="5" t="n">
-        <v>292</v>
+        <v>264</v>
       </c>
       <c r="I11" s="5" t="n">
         <v>65</v>
@@ -851,9 +851,9 @@
           <t>36/373</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>0/292</t>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>31/292</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -870,7 +870,7 @@
         <v>337</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>292</v>
+        <v>261</v>
       </c>
       <c r="I12" s="5" t="n">
         <v>65</v>
@@ -893,9 +893,9 @@
           <t>30/373</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>0/292</t>
+      <c r="D13" s="6" t="inlineStr">
+        <is>
+          <t>29/292</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -912,7 +912,7 @@
         <v>343</v>
       </c>
       <c r="H13" s="5" t="n">
-        <v>292</v>
+        <v>263</v>
       </c>
       <c r="I13" s="5" t="n">
         <v>65</v>
@@ -1148,7 +1148,7 @@
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="50" customWidth="1" min="2" max="2"/>
     <col width="50" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
     <col width="50" customWidth="1" min="5" max="5"/>
     <col width="50" customWidth="1" min="6" max="6"/>
   </cols>
@@ -1208,7 +1208,11 @@
           <t>9.3.6.5, 9.3.7.10, 9.3.7.2, 9.3.7.6, 9.3.7.7</t>
         </is>
       </c>
-      <c r="D3" s="16" t="inlineStr"/>
+      <c r="D3" s="16" t="inlineStr">
+        <is>
+          <t>7.EE.A.1.A, 8.EE.A.8, 8.EE.B.7, 8.G.2, see ebook</t>
+        </is>
+      </c>
       <c r="E3" s="17" t="inlineStr">
         <is>
           <t>TF: 1-10, 11, 26, 29-32, 42-44, (45); Team: 1-27, 28, 33 (LL); IS: eBook Scavenger Hunt Desmos
@@ -1245,7 +1249,11 @@
           <t>9.3.5.6, 9.3.5.7, 9.3.5.8, 9.3.6.2, 9.3.6.3, 9.3.6.5, 9.3.7.1, 9.3.7.2, 9.3.7.3</t>
         </is>
       </c>
-      <c r="D5" s="16" t="inlineStr"/>
+      <c r="D5" s="16" t="inlineStr">
+        <is>
+          <t>7.EE.4a, 7.EE.A.1.A, 7.EE.A.1.B, 7.SP.8a, 7.Sp.8a, 8.EE.C.7.A, see ebook</t>
+        </is>
+      </c>
       <c r="E5" s="17" t="inlineStr">
         <is>
           <t>TF: 2-13 to 15, 31-33, 43-45, (48-49), 65-66, (67); Team: 2-(34), 46, 47, 68 (LL); IS: Factoring: CC</t>
@@ -1281,7 +1289,11 @@
           <t>9.3.5.7, 9.3.5.8, 9.3.6.1, 9.3.6.4, 9.3.7.1</t>
         </is>
       </c>
-      <c r="D7" s="16" t="inlineStr"/>
+      <c r="D7" s="16" t="inlineStr">
+        <is>
+          <t>7.EE.3, 7.EE.4b, 7.SP.8a, 8.EE.C.7.A</t>
+        </is>
+      </c>
       <c r="E7" s="17" t="inlineStr">
         <is>
           <t>TF: 3-2, 3, 13-19, 42-43; Team: 3-4 (LL), 22, 41, 44; IS: Function Notation: CP 3B
@@ -1318,7 +1330,11 @@
           <t>9.3.7.1</t>
         </is>
       </c>
-      <c r="D9" s="16" t="inlineStr"/>
+      <c r="D9" s="16" t="inlineStr">
+        <is>
+          <t>8.EE.C.7.A</t>
+        </is>
+      </c>
       <c r="E9" s="17" t="inlineStr">
         <is>
           <t>TF: 4-1, 4, 18-19, 36-37, (38), (48); Team: 4-5, 6 (LL), 20-21, 39 (LL), 50 (LL); IS: Solution of Li</t>
@@ -1354,7 +1370,11 @@
           <t>9.3.5.9, 9.3.7.9</t>
         </is>
       </c>
-      <c r="D11" s="16" t="inlineStr"/>
+      <c r="D11" s="16" t="inlineStr">
+        <is>
+          <t>8.G.C.1</t>
+        </is>
+      </c>
       <c r="E11" s="17" t="inlineStr">
         <is>
           <t xml:space="preserve">TF: 5-(4 to 5), 18 to 23, 40 to 43; Team: 5-6, 7 (LL), 44, 47 (LL), 49 (Checkpoint 5A); IS: Line of </t>
@@ -1390,7 +1410,11 @@
           <t>9.3.6.5</t>
         </is>
       </c>
-      <c r="D13" s="16" t="inlineStr"/>
+      <c r="D13" s="16" t="inlineStr">
+        <is>
+          <t>see ebook</t>
+        </is>
+      </c>
       <c r="E13" s="17" t="inlineStr">
         <is>
           <t xml:space="preserve">TF: 6-1, 6-6, 6-16 to 6-17, 6-30 to 6-33 (consider use of 3-D Plotter eTool), 6-45 to 6-46, 6-60 to </t>
@@ -1483,7 +1507,11 @@
           <t>9.3.7.1, 9.3.7.2, 9.3.7.3</t>
         </is>
       </c>
-      <c r="D18" s="16" t="inlineStr"/>
+      <c r="D18" s="16" t="inlineStr">
+        <is>
+          <t>7.EE.A.1.A, 7.EE.A.1.B, 8.EE.C.7.A</t>
+        </is>
+      </c>
       <c r="E18" s="17" t="inlineStr">
         <is>
           <t xml:space="preserve">TF: 1-79 to 81, 98-101, 111; Team: 1-83, 102, 103 (LL); IS: Quadratic Formula: CCA PG 9.1
@@ -1512,7 +1540,11 @@
           <t>9.2.3.7, 9.3.5.6, 9.3.7.1</t>
         </is>
       </c>
-      <c r="D19" s="16" t="inlineStr"/>
+      <c r="D19" s="16" t="inlineStr">
+        <is>
+          <t>7.Sp.8a, 8.EE.C.7.A</t>
+        </is>
+      </c>
       <c r="E19" s="17" t="inlineStr">
         <is>
           <t>TF: 4-62, 80; Team: 4-63, 64 (LL), (82); IS: Solving for a Variable: CP 4B
@@ -1542,7 +1574,11 @@
           <t>9.3.7.3, 9.3.7.9</t>
         </is>
       </c>
-      <c r="D20" s="16" t="inlineStr"/>
+      <c r="D20" s="16" t="inlineStr">
+        <is>
+          <t>7.EE.A.1.B, 8.G.C.1</t>
+        </is>
+      </c>
       <c r="E20" s="17" t="inlineStr">
         <is>
           <t>TF: 5-(55 to 56), 58, 69, 70, 81, 82 (Further Guidance, as needed), 93, 94 (Desmos eTool); Team: 5-6</t>
@@ -1571,7 +1607,11 @@
           <t>9.3.7.2, 9.3.7.7</t>
         </is>
       </c>
-      <c r="D21" s="16" t="inlineStr"/>
+      <c r="D21" s="16" t="inlineStr">
+        <is>
+          <t>7.EE.A.1.A, 8.EE.A.8</t>
+        </is>
+      </c>
       <c r="E21" s="17" t="inlineStr">
         <is>
           <t>TF: 8-1, 8-2, 8-3 through 8-6 as needed, 8-28 through 8-30, 8-33, 8-34 or 8-35, 8-47 b through 8-52;</t>
@@ -1599,7 +1639,11 @@
           <t>9.3.5.3, 9.3.6.5</t>
         </is>
       </c>
-      <c r="D22" s="16" t="inlineStr"/>
+      <c r="D22" s="16" t="inlineStr">
+        <is>
+          <t>7.SP.8b, see ebook</t>
+        </is>
+      </c>
       <c r="E22" s="17" t="inlineStr">
         <is>
           <t xml:space="preserve">TF: 8-63 through 8-68, 8-81 through 8-82 (use FG as needed), 8-86, 8-100 through 8-102; Team: 8-69, </t>
@@ -1656,7 +1700,11 @@
           <t>9.1.1.1, 9.1.1.12, 9.1.1.14, 9.1.1.15, 9.1.1.2, 9.1.1.3, 9.1.1.4, 9.1.1.5</t>
         </is>
       </c>
-      <c r="D25" s="16" t="inlineStr"/>
+      <c r="D25" s="16" t="inlineStr">
+        <is>
+          <t>6.EE.A.2.A, 6.EE.A.2.B, 6.EE.A.3, 6.NS.B.4, 6.NS.C.6.C, 6.NS.C.7.C, MP 1, MP 7</t>
+        </is>
+      </c>
       <c r="E25" s="17" t="inlineStr">
         <is>
           <t>TF: 9-1 through 9-6, 9-31 through 9-34; Team: 9-35 (LL)</t>
@@ -1686,7 +1734,11 @@
           <t>9.1.1.5</t>
         </is>
       </c>
-      <c r="D26" s="16" t="inlineStr"/>
+      <c r="D26" s="16" t="inlineStr">
+        <is>
+          <t>6.EE.A.3</t>
+        </is>
+      </c>
       <c r="E26" s="17" t="inlineStr">
         <is>
           <t>Team: 9-61 (LL)</t>
@@ -1710,7 +1762,11 @@
           <t>9.1.1.10, 9.1.1.13, 9.1.1.7, 9.1.1.9</t>
         </is>
       </c>
-      <c r="D27" s="16" t="inlineStr"/>
+      <c r="D27" s="16" t="inlineStr">
+        <is>
+          <t>6.NS.C.6.A, 6.NS.C.7.A, 6.NS.C.7.B, 6.NS.C.7.D</t>
+        </is>
+      </c>
       <c r="E27" s="17" t="inlineStr">
         <is>
           <t>TF: 9-70 through 9-72; Team: 9-74 (LL)</t>
@@ -1767,7 +1823,11 @@
           <t>9.3.7.4, 9.3.7.5, 9.3.7.8</t>
         </is>
       </c>
-      <c r="D30" s="16" t="inlineStr"/>
+      <c r="D30" s="16" t="inlineStr">
+        <is>
+          <t>7.EE.B.4.B, 8.EE.B.8, 8.G.B.1</t>
+        </is>
+      </c>
       <c r="E30" s="17" t="inlineStr">
         <is>
           <t>TF: 10-72, 10-77 with FG as needed, 10-81, 10-105 to 10-106 with FG as needed,; Team: 10-86 LL, 10-9</t>
@@ -1792,7 +1852,11 @@
           <t>9.1.2.6, 9.3.7.8</t>
         </is>
       </c>
-      <c r="D31" s="16" t="inlineStr"/>
+      <c r="D31" s="16" t="inlineStr">
+        <is>
+          <t>8.G.B.1</t>
+        </is>
+      </c>
       <c r="E31" s="17" t="inlineStr">
         <is>
           <t>TF: 10-133 to 10-134, 10-135 to 10-141 with FG as needed, 10-164 to 10-167; Team: 10-144 (LL), 10-17</t>
@@ -1821,7 +1885,11 @@
           <t>9.3.5.7, 9.3.5.8</t>
         </is>
       </c>
-      <c r="D32" s="16" t="inlineStr"/>
+      <c r="D32" s="16" t="inlineStr">
+        <is>
+          <t>7.SP.8a</t>
+        </is>
+      </c>
       <c r="E32" s="17" t="inlineStr">
         <is>
           <t>TF: 3-57, (58 to 61), 73-74, 86-88, 99-100, 110-111; Team: 3-(62), 76, 77 (LL), 85, 89 (LL), 101 (LL</t>
@@ -1850,7 +1918,11 @@
           <t>9.3.7.1</t>
         </is>
       </c>
-      <c r="D33" s="16" t="inlineStr"/>
+      <c r="D33" s="16" t="inlineStr">
+        <is>
+          <t>8.EE.C.7.A</t>
+        </is>
+      </c>
       <c r="E33" s="17" t="inlineStr">
         <is>
           <t>TF: 6-89 to 6-93, 6-104 to 6-106, 6-123 &amp; 6-125; Team: 6-107 to 6-108, 6-113, 6-127, 6-130, 6-138 to</t>
@@ -1886,7 +1958,11 @@
           <t>9.1.2.4</t>
         </is>
       </c>
-      <c r="D35" s="16" t="inlineStr"/>
+      <c r="D35" s="16" t="inlineStr">
+        <is>
+          <t>6.RP.3c</t>
+        </is>
+      </c>
       <c r="E35" s="17" t="inlineStr">
         <is>
           <t>TF: 11-14 to 11-17 (11-16, FG, if needed), 11-28 with Reeses Pieces Applet; Team: 11-6 to 11-7, 11-1</t>
@@ -1915,7 +1991,11 @@
           <t>9.1.1.8</t>
         </is>
       </c>
-      <c r="D36" s="16" t="inlineStr"/>
+      <c r="D36" s="16" t="inlineStr">
+        <is>
+          <t>6.NS.C.6.B</t>
+        </is>
+      </c>
       <c r="E36" s="17" t="inlineStr">
         <is>
           <t>TF: 11-37 to 11-39, 11-50, 11-61, 11-63, 11-72 to 11-74; Team: 11-40 (LL), 11-41 to 11-43, 11-47, 11</t>
@@ -1971,7 +2051,11 @@
           <t>9.3.7.9</t>
         </is>
       </c>
-      <c r="D39" s="16" t="inlineStr"/>
+      <c r="D39" s="16" t="inlineStr">
+        <is>
+          <t>8.G.C.1</t>
+        </is>
+      </c>
       <c r="E39" s="17" t="inlineStr"/>
       <c r="F39" s="17" t="inlineStr"/>
     </row>
@@ -2007,7 +2091,11 @@
           <t>9.3.6.3, 9.3.7.10, 9.3.7.2, 9.3.7.3, 9.3.7.6</t>
         </is>
       </c>
-      <c r="D41" s="16" t="inlineStr"/>
+      <c r="D41" s="16" t="inlineStr">
+        <is>
+          <t>7.EE.4a, 7.EE.A.1.A, 7.EE.A.1.B, 8.EE.B.7, 8.G.2</t>
+        </is>
+      </c>
       <c r="E41" s="17" t="inlineStr">
         <is>
           <t>TF: 2-77 to 79, 104, 121-123, 153-160; Team: 2-106 (LL), 124 (LL), 161 (LL); IS: Exponent Rules: CCA</t>
@@ -2036,7 +2124,7 @@
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="50" customWidth="1" min="2" max="2"/>
     <col width="50" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
     <col width="50" customWidth="1" min="5" max="5"/>
     <col width="50" customWidth="1" min="6" max="6"/>
   </cols>
@@ -2119,7 +2207,11 @@
           <t>9.2.4.12, 9.2.4.6</t>
         </is>
       </c>
-      <c r="D5" s="16" t="inlineStr"/>
+      <c r="D5" s="16" t="inlineStr">
+        <is>
+          <t>7.RP.A.2.D, 7.SP.7a</t>
+        </is>
+      </c>
       <c r="E5" s="17" t="inlineStr">
         <is>
           <t>TF: 1-(1,2, 1-8 to 13, 1-30, 31), 1-37 to 40; Team: 1-19 to 24; IS: 1-(41)</t>
@@ -2148,7 +2240,11 @@
           <t>9.2.4.1, 9.2.4.12, 9.2.4.13, 9.2.4.14</t>
         </is>
       </c>
-      <c r="D6" s="16" t="inlineStr"/>
+      <c r="D6" s="16" t="inlineStr">
+        <is>
+          <t>7.NS.A.1.A, 7.SP.7a, 7.SP.7b, 7.SP.7c</t>
+        </is>
+      </c>
       <c r="E6" s="17" t="inlineStr">
         <is>
           <t>TF: 1-(59 to 60), 61, (68 to 73), 81 to 82, 90, (91), 93; Team: 1-(47 to 49), 50-51, (52), 62, 83, (</t>
@@ -2183,7 +2279,11 @@
           <t>9.2.4.1, 9.2.4.12, 9.2.4.7</t>
         </is>
       </c>
-      <c r="D8" s="16" t="inlineStr"/>
+      <c r="D8" s="16" t="inlineStr">
+        <is>
+          <t>7.NS.A.1.A, 7.RP.A.2.B, 7.SP.7a</t>
+        </is>
+      </c>
       <c r="E8" s="17" t="inlineStr">
         <is>
           <t>TF: 2-(1), 14, 15, (28), 37, 46, 47, (50-52,54); Team: 2-2 to 4, 16-18, 25, (29), 40, 48, 49, 53; IS</t>
@@ -2212,7 +2312,11 @@
           <t>9.2.3.6, 9.2.4.12</t>
         </is>
       </c>
-      <c r="D9" s="16" t="inlineStr"/>
+      <c r="D9" s="16" t="inlineStr">
+        <is>
+          <t>5.NF.A.1, 7.SP.7a</t>
+        </is>
+      </c>
       <c r="E9" s="17" t="inlineStr">
         <is>
           <t xml:space="preserve">TF: 2-(60 to 63), 70, 79-80, (81), 82, 90 to 92; Team: 2-71,(72), 83, (84); IS: 2-(64), 73 (LL), 93 </t>
@@ -2248,7 +2352,11 @@
           <t>9.2.3.9</t>
         </is>
       </c>
-      <c r="D11" s="16" t="inlineStr"/>
+      <c r="D11" s="16" t="inlineStr">
+        <is>
+          <t>7.NS.A.1.D</t>
+        </is>
+      </c>
       <c r="E11" s="17" t="inlineStr">
         <is>
           <t>TF: 3-1,(2), 24, (35), 36-37; Team: 3-(11), 13, (15), 26-27, 38-39; IS: 3-(3), 4 (LL), 12,(14),16,17</t>
@@ -2284,7 +2392,11 @@
           <t>9.2.3.3, 9.2.3.8, 9.2.4.12</t>
         </is>
       </c>
-      <c r="D13" s="16" t="inlineStr"/>
+      <c r="D13" s="16" t="inlineStr">
+        <is>
+          <t>7.SP.7a, 7.SP.C.7.B, 7.SP.C.8.A</t>
+        </is>
+      </c>
       <c r="E13" s="17" t="inlineStr">
         <is>
           <t>TF: 4-1 to 4, (23-25), 45, 46; Team: 4-5, 13-16, 33-36; IS: 4-12, 26 (LL), 37, 38 (LL)</t>
@@ -2316,7 +2428,11 @@
           <t>9.2.3.3, 9.2.3.8</t>
         </is>
       </c>
-      <c r="D15" s="16" t="inlineStr"/>
+      <c r="D15" s="16" t="inlineStr">
+        <is>
+          <t>7.SP.C.7.B, 7.SP.C.8.A</t>
+        </is>
+      </c>
       <c r="E15" s="17" t="inlineStr"/>
       <c r="F15" s="17" t="inlineStr">
         <is>
@@ -2336,7 +2452,11 @@
           <t>9.1.2.8, 9.2.3.2, 9.2.3.3</t>
         </is>
       </c>
-      <c r="D16" s="16" t="inlineStr"/>
+      <c r="D16" s="16" t="inlineStr">
+        <is>
+          <t>7.NS.A.2.D, 7.SP.C.7.B, 7.SP.C.8.C</t>
+        </is>
+      </c>
       <c r="E16" s="17" t="inlineStr"/>
       <c r="F16" s="17" t="inlineStr"/>
     </row>
@@ -2352,7 +2472,11 @@
           <t>9.2.3.2, 9.2.3.3</t>
         </is>
       </c>
-      <c r="D17" s="16" t="inlineStr"/>
+      <c r="D17" s="16" t="inlineStr">
+        <is>
+          <t>7.NS.A.2.D, 7.SP.C.7.B</t>
+        </is>
+      </c>
       <c r="E17" s="17" t="inlineStr"/>
       <c r="F17" s="17" t="inlineStr"/>
     </row>
@@ -2375,7 +2499,11 @@
           <t>9.2.4.10, 9.2.4.4, 9.2.4.5, 9.2.4.7</t>
         </is>
       </c>
-      <c r="D19" s="16" t="inlineStr"/>
+      <c r="D19" s="16" t="inlineStr">
+        <is>
+          <t>7.NS.A.2.C, 7.RP.3, 7.RP.A.2.A, 7.RP.A.2.B</t>
+        </is>
+      </c>
       <c r="E19" s="17" t="inlineStr"/>
       <c r="F19" s="17" t="inlineStr">
         <is>
@@ -2395,7 +2523,11 @@
           <t>9.2.3.1, 9.2.4.10</t>
         </is>
       </c>
-      <c r="D20" s="16" t="inlineStr"/>
+      <c r="D20" s="16" t="inlineStr">
+        <is>
+          <t>7.RP.3, 8.EE.C.7.B</t>
+        </is>
+      </c>
       <c r="E20" s="17" t="inlineStr"/>
       <c r="F20" s="17" t="inlineStr">
         <is>
@@ -2426,7 +2558,11 @@
           <t>9.1.2.1, 9.1.2.2, 9.1.2.3, 9.1.2.4, 9.1.2.7</t>
         </is>
       </c>
-      <c r="D22" s="16" t="inlineStr"/>
+      <c r="D22" s="16" t="inlineStr">
+        <is>
+          <t>6.EE.A.2.C, 6.EE.A.4, 6.G.1, 6.RP.3c, Review skills needed for 6.NS.1</t>
+        </is>
+      </c>
       <c r="E22" s="17" t="inlineStr">
         <is>
           <t>TF: 4-53 to 56, (57), 65-66, (67), (75-79), (87-94), 101-102, (105); Team: 4-64, 103, 104, (106-107)</t>
@@ -2451,7 +2587,11 @@
           <t>9.2.4.15</t>
         </is>
       </c>
-      <c r="D23" s="16" t="inlineStr"/>
+      <c r="D23" s="16" t="inlineStr">
+        <is>
+          <t>7.SP.6</t>
+        </is>
+      </c>
       <c r="E23" s="17" t="inlineStr"/>
       <c r="F23" s="17" t="inlineStr">
         <is>
@@ -2471,7 +2611,11 @@
           <t>9.2.4.3, 9.2.4.4, 9.2.4.7</t>
         </is>
       </c>
-      <c r="D24" s="16" t="inlineStr"/>
+      <c r="D24" s="16" t="inlineStr">
+        <is>
+          <t>7.NS.A.2.A, 7.NS.A.2.C, 7.RP.A.2.B</t>
+        </is>
+      </c>
       <c r="E24" s="17" t="inlineStr"/>
       <c r="F24" s="17" t="inlineStr">
         <is>
@@ -2491,7 +2635,11 @@
           <t>9.2.3.1</t>
         </is>
       </c>
-      <c r="D25" s="16" t="inlineStr"/>
+      <c r="D25" s="16" t="inlineStr">
+        <is>
+          <t>8.EE.C.7.B</t>
+        </is>
+      </c>
       <c r="E25" s="17" t="inlineStr"/>
       <c r="F25" s="17" t="inlineStr">
         <is>
@@ -2546,7 +2694,11 @@
           <t>9.2.4.10, 9.2.4.11, 9.2.4.12, 9.2.4.4, 9.2.4.6, 9.2.4.7</t>
         </is>
       </c>
-      <c r="D28" s="16" t="inlineStr"/>
+      <c r="D28" s="16" t="inlineStr">
+        <is>
+          <t>7.NS.A.2.C, 7.RP.3, 7.RP.A.2.B, 7.RP.A.2.D, 7.SP.7a</t>
+        </is>
+      </c>
       <c r="E28" s="17" t="inlineStr">
         <is>
           <t xml:space="preserve">TF: 3-47, 48, 50, 59, 60, 74, (82-86), 105-106, (107); Team: 3-49, (51), 61, 62, 71, 72, 94-96; IS: </t>
@@ -2571,7 +2723,11 @@
           <t>9.2.3.3, 9.2.4.1, 9.2.4.12, 9.2.4.15, 9.2.4.3</t>
         </is>
       </c>
-      <c r="D29" s="16" t="inlineStr"/>
+      <c r="D29" s="16" t="inlineStr">
+        <is>
+          <t>7.NS.A.1.A, 7.NS.A.2.A, 7.SP.6, 7.SP.7a, 7.SP.C.7.B</t>
+        </is>
+      </c>
       <c r="E29" s="17" t="inlineStr">
         <is>
           <t>IS: This chapter also begins a slight increase in the number of and difficulty level of the homework</t>
@@ -2595,7 +2751,11 @@
           <t>9.2.3.9</t>
         </is>
       </c>
-      <c r="D30" s="16" t="inlineStr"/>
+      <c r="D30" s="16" t="inlineStr">
+        <is>
+          <t>7.NS.A.1.D</t>
+        </is>
+      </c>
       <c r="E30" s="17" t="inlineStr"/>
       <c r="F30" s="17" t="inlineStr">
         <is>
@@ -2615,7 +2775,11 @@
           <t>9.2.4.3</t>
         </is>
       </c>
-      <c r="D31" s="16" t="inlineStr"/>
+      <c r="D31" s="16" t="inlineStr">
+        <is>
+          <t>7.NS.A.2.A</t>
+        </is>
+      </c>
       <c r="E31" s="17" t="inlineStr"/>
       <c r="F31" s="17" t="inlineStr">
         <is>
@@ -2646,7 +2810,11 @@
           <t>9.2.3.3, 9.2.4.12</t>
         </is>
       </c>
-      <c r="D33" s="16" t="inlineStr"/>
+      <c r="D33" s="16" t="inlineStr">
+        <is>
+          <t>7.SP.7a, 7.SP.C.7.B</t>
+        </is>
+      </c>
       <c r="E33" s="17" t="inlineStr">
         <is>
           <t>TF: 2-(99), 101, (109); Team: 2- 100,102, 111, 112; IS: 2-103, 110 (LL)</t>
@@ -2671,7 +2839,11 @@
           <t>9.2.3.4, 9.2.3.9</t>
         </is>
       </c>
-      <c r="D34" s="16" t="inlineStr"/>
+      <c r="D34" s="16" t="inlineStr">
+        <is>
+          <t>7.NS.A.1.D, 7.SP.C.7.A</t>
+        </is>
+      </c>
       <c r="E34" s="17" t="inlineStr"/>
       <c r="F34" s="17" t="inlineStr">
         <is>
@@ -2691,7 +2863,11 @@
           <t>9.2.4.1, 9.2.4.12</t>
         </is>
       </c>
-      <c r="D35" s="16" t="inlineStr"/>
+      <c r="D35" s="16" t="inlineStr">
+        <is>
+          <t>7.NS.A.1.A, 7.SP.7a</t>
+        </is>
+      </c>
       <c r="E35" s="17" t="inlineStr"/>
       <c r="F35" s="17" t="inlineStr">
         <is>
@@ -2718,7 +2894,11 @@
           <t>9.2.4.8, 9.2.4.9</t>
         </is>
       </c>
-      <c r="D37" s="16" t="inlineStr"/>
+      <c r="D37" s="16" t="inlineStr">
+        <is>
+          <t>7.NS.A.1.C, 7.RP.A.2.C</t>
+        </is>
+      </c>
       <c r="E37" s="17" t="inlineStr"/>
       <c r="F37" s="17" t="inlineStr">
         <is>
@@ -2738,7 +2918,11 @@
           <t>9.1.2.1, 9.1.2.3, 9.1.2.5</t>
         </is>
       </c>
-      <c r="D38" s="16" t="inlineStr"/>
+      <c r="D38" s="16" t="inlineStr">
+        <is>
+          <t>6.EE.A.4, 6.NS.3, Review skills needed for 6.NS.1</t>
+        </is>
+      </c>
       <c r="E38" s="17" t="inlineStr"/>
       <c r="F38" s="17" t="inlineStr">
         <is>
@@ -2758,7 +2942,11 @@
           <t>9.1.2.1</t>
         </is>
       </c>
-      <c r="D39" s="16" t="inlineStr"/>
+      <c r="D39" s="16" t="inlineStr">
+        <is>
+          <t>6.EE.A.4</t>
+        </is>
+      </c>
       <c r="E39" s="17" t="inlineStr"/>
       <c r="F39" s="17" t="inlineStr">
         <is>
@@ -2785,7 +2973,11 @@
           <t>9.2.3.4, 9.2.3.5</t>
         </is>
       </c>
-      <c r="D41" s="16" t="inlineStr"/>
+      <c r="D41" s="16" t="inlineStr">
+        <is>
+          <t>7.SP.C.7.A, Prep for 7.SP.C.8.A</t>
+        </is>
+      </c>
       <c r="E41" s="17" t="inlineStr"/>
       <c r="F41" s="17" t="inlineStr">
         <is>
@@ -2805,7 +2997,11 @@
           <t>9.2.3.5, 9.2.4.12, 9.2.4.8, 9.2.4.9</t>
         </is>
       </c>
-      <c r="D42" s="16" t="inlineStr"/>
+      <c r="D42" s="16" t="inlineStr">
+        <is>
+          <t>7.NS.A.1.C, 7.RP.A.2.C, 7.SP.7a, Prep for 7.SP.C.8.A</t>
+        </is>
+      </c>
       <c r="E42" s="17" t="inlineStr"/>
       <c r="F42" s="17" t="inlineStr">
         <is>
@@ -2832,7 +3028,11 @@
           <t>9.2.3.3, 9.2.4.12, 9.3.6.6</t>
         </is>
       </c>
-      <c r="D44" s="16" t="inlineStr"/>
+      <c r="D44" s="16" t="inlineStr">
+        <is>
+          <t>7.SP.7a, 7.SP.C.7.B, MP4</t>
+        </is>
+      </c>
       <c r="E44" s="17" t="inlineStr"/>
       <c r="F44" s="17" t="inlineStr">
         <is>
@@ -41119,11 +41319,11 @@
         </is>
       </c>
       <c r="G160" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H160" s="8" t="inlineStr">
         <is>
-          <t>6.1.1.4 (MN-2022)</t>
+          <t>6.4.1.1 (MN-2007), 6.4.1.2 (MN-2007), 6.1.1.4 (MN-2022)</t>
         </is>
       </c>
     </row>
@@ -41153,11 +41353,11 @@
         </is>
       </c>
       <c r="G161" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H161" s="8" t="inlineStr">
         <is>
-          <t>6.G.A.1 (CCSS-M), 6.2.3.5 (MN-2022)</t>
+          <t>6.G.A.1 (CCSS-M), 6.3.1.1 (MN-2007), 6.3.1.2 (MN-2007), 6.3.2.1 (MN-2007), 6.2.3.5 (MN-2022)</t>
         </is>
       </c>
     </row>
@@ -41221,11 +41421,11 @@
         </is>
       </c>
       <c r="G163" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H163" s="8" t="inlineStr">
         <is>
-          <t>6.SP.B.4 (CCSS-M), 6.1.1.1 (MN-2022), 6.1.1.4 (MN-2022), 6.1.1.5 (MN-2022)</t>
+          <t>6.SP.B.4 (CCSS-M), 6.4.1.1 (MN-2007), 6.4.1.2 (MN-2007), 6.1.1.1 (MN-2022), 6.1.1.4 (MN-2022), 6.1.1.5 (MN-2022)</t>
         </is>
       </c>
     </row>
@@ -41383,11 +41583,11 @@
         </is>
       </c>
       <c r="G168" t="n">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="H168" s="8" t="inlineStr">
         <is>
-          <t>6.EE.A.1 (CCSS-M), 6.3.5.4 (MN-2022), 6.NS.B.4 (CCSS-M), 6.EE.A.2.B (CCSS-M)</t>
+          <t>6.EE.A.1 (CCSS-M), 6.2.1.1 (MN-2007), 6.2.2.1 (MN-2007), 6.2.2.2 (MN-2007), 6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.1.3.1 (MN-2007), 6.1.3.2 (MN-2007), 6.1.3.3 (MN-2007) +7 more</t>
         </is>
       </c>
     </row>
@@ -41417,11 +41617,11 @@
         </is>
       </c>
       <c r="G169" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="H169" s="8" t="inlineStr">
         <is>
-          <t>6.SP.B.4 (CCSS-M), 6.1.1.4 (MN-2022), 6.2.3.5 (MN-2022)</t>
+          <t>6.3.1.1 (MN-2007), 6.3.1.2 (MN-2007), 6.3.2.1 (MN-2007), 6.SP.B.4 (CCSS-M), 6.4.1.1 (MN-2007), 6.4.1.2 (MN-2007), 6.1.1.4 (MN-2022), 6.2.3.5 (MN-2022)</t>
         </is>
       </c>
     </row>
@@ -41451,11 +41651,11 @@
         </is>
       </c>
       <c r="G170" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H170" s="8" t="inlineStr">
         <is>
-          <t>6.SP.B.4 (CCSS-M), 6.1.1.4 (MN-2022)</t>
+          <t>6.SP.B.4 (CCSS-M), 6.4.1.1 (MN-2007), 6.4.1.2 (MN-2007), 6.1.1.4 (MN-2022)</t>
         </is>
       </c>
     </row>
@@ -41519,11 +41719,11 @@
         </is>
       </c>
       <c r="G172" t="n">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="H172" s="8" t="inlineStr">
         <is>
-          <t>6.G.A.1 (CCSS-M), 6.3.6.1 (MN-2022)</t>
+          <t>6.G.A.1 (CCSS-M), 6.2.1.1 (MN-2007), 6.2.2.1 (MN-2007), 6.2.2.2 (MN-2007), 6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.1.3.1 (MN-2007), 6.1.3.2 (MN-2007), 6.1.3.3 (MN-2007) +5 more</t>
         </is>
       </c>
     </row>
@@ -41553,11 +41753,11 @@
         </is>
       </c>
       <c r="G173" t="n">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="H173" s="8" t="inlineStr">
         <is>
-          <t>6.G.A.1 (CCSS-M), 6.3.5.5 (MN-2022)</t>
+          <t>6.G.A.1 (CCSS-M), 6.2.1.1 (MN-2007), 6.2.2.1 (MN-2007), 6.2.2.2 (MN-2007), 6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.1.3.1 (MN-2007), 6.1.3.2 (MN-2007), 6.1.3.3 (MN-2007) +5 more</t>
         </is>
       </c>
     </row>
@@ -41723,11 +41923,11 @@
         </is>
       </c>
       <c r="G178" t="n">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="H178" s="8" t="inlineStr">
         <is>
-          <t>6.3.5.5 (MN-2022), 6.RP.A.3.C (CCSS-M)</t>
+          <t>6.2.1.1 (MN-2007), 6.2.2.1 (MN-2007), 6.2.2.2 (MN-2007), 6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.1.3.1 (MN-2007), 6.1.3.2 (MN-2007), 6.1.3.3 (MN-2007), 6.1.1.4 (MN-2007) +5 more</t>
         </is>
       </c>
     </row>
@@ -41757,11 +41957,11 @@
         </is>
       </c>
       <c r="G179" t="n">
-        <v>3</v>
+        <v>16</v>
       </c>
       <c r="H179" s="8" t="inlineStr">
         <is>
-          <t>6.3.5.11 (MN-2022), 6.3.6.6 (MN-2022), 6.RP.A.3.C (CCSS-M)</t>
+          <t>6.2.1.1 (MN-2007), 6.2.2.1 (MN-2007), 6.2.2.2 (MN-2007), 6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.1.3.1 (MN-2007), 6.1.3.2 (MN-2007), 6.1.3.3 (MN-2007), 6.1.1.4 (MN-2007) +6 more</t>
         </is>
       </c>
     </row>
@@ -41791,11 +41991,11 @@
         </is>
       </c>
       <c r="G180" t="n">
-        <v>3</v>
+        <v>16</v>
       </c>
       <c r="H180" s="8" t="inlineStr">
         <is>
-          <t>6.NS.B.3 (CCSS-M), 6.3.5.11 (MN-2022), 6.3.6.2 (MN-2022)</t>
+          <t>6.2.1.1 (MN-2007), 6.2.2.1 (MN-2007), 6.2.2.2 (MN-2007), 6.NS.B.3 (CCSS-M), 6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.1.3.1 (MN-2007), 6.1.3.2 (MN-2007), 6.1.3.3 (MN-2007) +6 more</t>
         </is>
       </c>
     </row>
@@ -41859,11 +42059,11 @@
         </is>
       </c>
       <c r="G182" t="n">
-        <v>3</v>
+        <v>16</v>
       </c>
       <c r="H182" s="8" t="inlineStr">
         <is>
-          <t>6.NS.B.3 (CCSS-M), 6.3.6.2 (MN-2022), 6.RP.A.3.C (CCSS-M)</t>
+          <t>6.2.1.1 (MN-2007), 6.2.2.1 (MN-2007), 6.2.2.2 (MN-2007), 6.NS.B.3 (CCSS-M), 6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.1.3.1 (MN-2007), 6.1.3.2 (MN-2007), 6.1.3.3 (MN-2007) +6 more</t>
         </is>
       </c>
     </row>
@@ -41893,11 +42093,11 @@
         </is>
       </c>
       <c r="G183" t="n">
-        <v>3</v>
+        <v>16</v>
       </c>
       <c r="H183" s="8" t="inlineStr">
         <is>
-          <t>6.RP.A.1 (CCSS-M), 6.3.5.2 (MN-2022), 6.3.6.5 (MN-2022)</t>
+          <t>6.2.1.1 (MN-2007), 6.2.2.1 (MN-2007), 6.2.2.2 (MN-2007), 6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.1.3.1 (MN-2007), 6.1.3.2 (MN-2007), 6.1.3.3 (MN-2007), 6.1.1.4 (MN-2007) +6 more</t>
         </is>
       </c>
     </row>
@@ -41927,11 +42127,11 @@
         </is>
       </c>
       <c r="G184" t="n">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="H184" s="8" t="inlineStr">
         <is>
-          <t>6.3.5.1 (MN-2022), 6.3.5.2 (MN-2022), 6.NS.C.6.A (CCSS-M), 6.NS.C.6.B (CCSS-M)</t>
+          <t>6.2.1.1 (MN-2007), 6.2.2.1 (MN-2007), 6.2.2.2 (MN-2007), 6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.1.3.1 (MN-2007), 6.1.3.2 (MN-2007), 6.1.3.3 (MN-2007), 6.1.1.4 (MN-2007) +7 more</t>
         </is>
       </c>
     </row>
@@ -41961,11 +42161,11 @@
         </is>
       </c>
       <c r="G185" t="n">
-        <v>6</v>
+        <v>19</v>
       </c>
       <c r="H185" s="8" t="inlineStr">
         <is>
-          <t>6.NS.C.5 (CCSS-M), 6.3.5.2 (MN-2022), 6.3.5.3 (MN-2022), 6.3.5.5 (MN-2022), 6.NS.C.6.A (CCSS-M), 6.NS.C.7.A (CCSS-M)</t>
+          <t>6.2.1.1 (MN-2007), 6.2.2.1 (MN-2007), 6.2.2.2 (MN-2007), 6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.NS.C.5 (CCSS-M), 6.1.3.1 (MN-2007), 6.1.3.2 (MN-2007), 6.1.3.3 (MN-2007) +9 more</t>
         </is>
       </c>
     </row>
@@ -41995,11 +42195,11 @@
         </is>
       </c>
       <c r="G186" t="n">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="H186" s="8" t="inlineStr">
         <is>
-          <t>6.3.5.3 (MN-2022), 6.3.5.6 (MN-2022), 6.NS.C.7.B (CCSS-M), 6.NS.C.7.C (CCSS-M), 6.NS.C.7.D (CCSS-M)</t>
+          <t>6.2.1.1 (MN-2007), 6.2.2.1 (MN-2007), 6.2.2.2 (MN-2007), 6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.1.3.1 (MN-2007), 6.1.3.2 (MN-2007), 6.1.3.3 (MN-2007), 6.1.1.4 (MN-2007) +8 more</t>
         </is>
       </c>
     </row>
@@ -42029,11 +42229,11 @@
         </is>
       </c>
       <c r="G187" t="n">
-        <v>7</v>
+        <v>23</v>
       </c>
       <c r="H187" s="8" t="inlineStr">
         <is>
-          <t>6.NS.C.8 (CCSS-M), 6.2.4.3 (MN-2022), 6.3.5.1 (MN-2022), 6.3.5.2 (MN-2022), 6.3.5.6 (MN-2022), 6.NS.C.6.B (CCSS-M), 6.NS.C.6.C (CCSS-M)</t>
+          <t>6.3.1.1 (MN-2007), 6.3.1.2 (MN-2007), 6.NS.C.8 (CCSS-M), 6.3.2.1 (MN-2007), 6.2.1.1 (MN-2007), 6.2.2.1 (MN-2007), 6.2.2.2 (MN-2007), 6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007) +13 more</t>
         </is>
       </c>
     </row>
@@ -42063,11 +42263,11 @@
         </is>
       </c>
       <c r="G188" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H188" s="8" t="inlineStr">
         <is>
-          <t>6.EE.B.6 (CCSS-M), 6.1.2.2 (MN-2022), 6.EE.A.2.A (CCSS-M)</t>
+          <t>6.EE.B.6 (CCSS-M), 6.4.1.1 (MN-2007), 6.4.1.2 (MN-2007), 6.1.2.2 (MN-2022), 6.EE.A.2.A (CCSS-M)</t>
         </is>
       </c>
     </row>
@@ -42131,11 +42331,11 @@
         </is>
       </c>
       <c r="G190" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H190" s="8" t="inlineStr">
         <is>
-          <t>6.EE.B.6 (CCSS-M), 6.1.2.1 (MN-2022), 6.EE.A.2.A (CCSS-M), 6.EE.A.4 (CCSS-M), 6.EE.A.2.C (CCSS-M)</t>
+          <t>6.EE.B.6 (CCSS-M), 6.4.1.1 (MN-2007), 6.4.1.2 (MN-2007), 6.1.2.1 (MN-2022), 6.EE.A.2.A (CCSS-M), 6.EE.A.4 (CCSS-M), 6.EE.A.2.C (CCSS-M)</t>
         </is>
       </c>
     </row>
@@ -42301,11 +42501,11 @@
         </is>
       </c>
       <c r="G195" t="n">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="H195" s="8" t="inlineStr">
         <is>
-          <t>6.3.6.3 (MN-2022), 6.3.6.4 (MN-2022), 6.3.7.1 (MN-2022), Review skills needed for 6.NS.1 (CCSS-M)</t>
+          <t>6.2.1.1 (MN-2007), 6.2.2.1 (MN-2007), 6.2.2.2 (MN-2007), 6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.1.3.1 (MN-2007), 6.1.3.2 (MN-2007), 6.1.3.3 (MN-2007), 6.1.1.4 (MN-2007) +7 more</t>
         </is>
       </c>
     </row>
@@ -42365,11 +42565,11 @@
         </is>
       </c>
       <c r="G197" t="n">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="H197" s="8" t="inlineStr">
         <is>
-          <t>6.3.6.3 (MN-2022), 6.3.6.4 (MN-2022), 6.3.7.1 (MN-2022), Review skills needed for 6.NS.1 (CCSS-M)</t>
+          <t>6.2.1.1 (MN-2007), 6.2.2.1 (MN-2007), 6.2.2.2 (MN-2007), 6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.1.3.1 (MN-2007), 6.1.3.2 (MN-2007), 6.1.3.3 (MN-2007), 6.1.1.4 (MN-2007) +7 more</t>
         </is>
       </c>
     </row>
@@ -42433,11 +42633,11 @@
         </is>
       </c>
       <c r="G199" t="n">
-        <v>3</v>
+        <v>16</v>
       </c>
       <c r="H199" s="8" t="inlineStr">
         <is>
-          <t>6.3.6.5 (MN-2022), 6.RP.3c (CCSS-M), 6.NS.3 (CCSS-M)</t>
+          <t>6.2.1.1 (MN-2007), 6.2.2.1 (MN-2007), 6.2.2.2 (MN-2007), 6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.1.3.1 (MN-2007), 6.1.3.2 (MN-2007), 6.1.3.3 (MN-2007), 6.1.1.4 (MN-2007) +6 more</t>
         </is>
       </c>
     </row>
@@ -42727,11 +42927,11 @@
         </is>
       </c>
       <c r="G208" t="n">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="H208" s="8" t="inlineStr">
         <is>
-          <t>6.3.5.7 (MN-2022)</t>
+          <t>6.2.1.1 (MN-2007), 6.2.2.1 (MN-2007), 6.2.2.2 (MN-2007), 6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.1.3.1 (MN-2007), 6.1.3.2 (MN-2007), 6.1.3.3 (MN-2007), 6.1.1.4 (MN-2007) +4 more</t>
         </is>
       </c>
     </row>
@@ -42761,11 +42961,11 @@
         </is>
       </c>
       <c r="G209" t="n">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="H209" s="8" t="inlineStr">
         <is>
-          <t>6.3.5.11 (MN-2022), 6.3.6.6 (MN-2022)</t>
+          <t>6.2.1.1 (MN-2007), 6.2.2.1 (MN-2007), 6.2.2.2 (MN-2007), 6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.1.3.1 (MN-2007), 6.1.3.2 (MN-2007), 6.1.3.3 (MN-2007), 6.1.1.4 (MN-2007) +5 more</t>
         </is>
       </c>
     </row>
@@ -42911,11 +43111,11 @@
       </c>
       <c r="F214" s="8" t="inlineStr"/>
       <c r="G214" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H214" s="8" t="inlineStr">
         <is>
-          <t>6.2.3.5 (MN-2022)</t>
+          <t>6.3.1.1 (MN-2007), 6.3.1.2 (MN-2007), 6.3.2.1 (MN-2007), 6.2.3.5 (MN-2022)</t>
         </is>
       </c>
     </row>
@@ -42945,11 +43145,11 @@
         </is>
       </c>
       <c r="G215" t="n">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H215" s="8" t="inlineStr">
         <is>
-          <t>6.1.2.1 (MN-2022), 6.1.2.2 (MN-2022), 6.1.2.3 (MN-2022), 6.3.5.11 (MN-2022)</t>
+          <t>6.2.1.1 (MN-2007), 6.2.2.1 (MN-2007), 6.2.2.2 (MN-2007), 6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.1.3.1 (MN-2007), 6.1.3.2 (MN-2007), 6.1.3.3 (MN-2007), 6.1.1.4 (MN-2007) +9 more</t>
         </is>
       </c>
     </row>
@@ -43031,11 +43231,11 @@
       <c r="E218" s="7" t="n"/>
       <c r="F218" s="8" t="inlineStr"/>
       <c r="G218" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H218" s="8" t="inlineStr">
         <is>
-          <t>6.1.2.3 (MN-2022)</t>
+          <t>6.4.1.1 (MN-2007), 6.4.1.2 (MN-2007), 6.1.2.3 (MN-2022)</t>
         </is>
       </c>
     </row>
@@ -43289,11 +43489,11 @@
         </is>
       </c>
       <c r="G227" t="n">
-        <v>2</v>
+        <v>17</v>
       </c>
       <c r="H227" s="8" t="inlineStr">
         <is>
-          <t>6.1.1.3 (MN-2022), 6.3.5.9 (MN-2022)</t>
+          <t>6.2.1.1 (MN-2007), 6.2.2.1 (MN-2007), 6.2.2.2 (MN-2007), 6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.1.3.1 (MN-2007), 6.1.3.2 (MN-2007), 6.1.3.3 (MN-2007), 6.1.1.4 (MN-2007) +7 more</t>
         </is>
       </c>
     </row>
@@ -43323,11 +43523,11 @@
         </is>
       </c>
       <c r="G228" t="n">
-        <v>3</v>
+        <v>18</v>
       </c>
       <c r="H228" s="8" t="inlineStr">
         <is>
-          <t>6.1.1.5 (MN-2022), 6.3.5.7 (MN-2022), 6.3.5.8 (MN-2022)</t>
+          <t>6.2.1.1 (MN-2007), 6.2.2.1 (MN-2007), 6.2.2.2 (MN-2007), 6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.1.3.1 (MN-2007), 6.1.3.2 (MN-2007), 6.1.3.3 (MN-2007), 6.1.1.4 (MN-2007) +8 more</t>
         </is>
       </c>
     </row>
@@ -43387,11 +43587,11 @@
         </is>
       </c>
       <c r="G230" t="n">
-        <v>3</v>
+        <v>21</v>
       </c>
       <c r="H230" s="8" t="inlineStr">
         <is>
-          <t>6.1.1.3 (MN-2022), 6.2.3.4 (MN-2022), 6.3.5.8 (MN-2022)</t>
+          <t>6.3.1.1 (MN-2007), 6.3.1.2 (MN-2007), 6.3.2.1 (MN-2007), 6.2.1.1 (MN-2007), 6.2.2.1 (MN-2007), 6.2.2.2 (MN-2007), 6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.1.3.1 (MN-2007) +11 more</t>
         </is>
       </c>
     </row>
@@ -43421,11 +43621,11 @@
         </is>
       </c>
       <c r="G231" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H231" s="8" t="inlineStr">
         <is>
-          <t>6.1.1.5 (MN-2022)</t>
+          <t>6.4.1.1 (MN-2007), 6.4.1.2 (MN-2007), 6.1.1.5 (MN-2022)</t>
         </is>
       </c>
     </row>
@@ -43455,11 +43655,11 @@
         </is>
       </c>
       <c r="G232" t="n">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="H232" s="8" t="inlineStr">
         <is>
-          <t>6.1.1.1 (MN-2022), 6.1.1.2 (MN-2022), 6.3.5.9 (MN-2022), 6.3.6.1 (MN-2022)</t>
+          <t>6.2.1.1 (MN-2007), 6.2.2.1 (MN-2007), 6.2.2.2 (MN-2007), 6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.1.3.1 (MN-2007), 6.1.3.2 (MN-2007), 6.1.3.3 (MN-2007), 6.1.1.4 (MN-2007) +9 more</t>
         </is>
       </c>
     </row>
@@ -43567,11 +43767,11 @@
         </is>
       </c>
       <c r="G236" t="n">
-        <v>3</v>
+        <v>19</v>
       </c>
       <c r="H236" s="8" t="inlineStr">
         <is>
-          <t>6.2.3.4 (MN-2022), 6.3.5.9 (MN-2022), 6.3.5.10 (MN-2022)</t>
+          <t>6.3.1.1 (MN-2007), 6.3.1.2 (MN-2007), 6.3.2.1 (MN-2007), 6.2.1.1 (MN-2007), 6.2.2.1 (MN-2007), 6.2.2.2 (MN-2007), 6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.1.3.1 (MN-2007) +9 more</t>
         </is>
       </c>
     </row>
@@ -43601,11 +43801,11 @@
         </is>
       </c>
       <c r="G237" t="n">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="H237" s="8" t="inlineStr">
         <is>
-          <t>6.3.5.9 (MN-2022)</t>
+          <t>6.2.1.1 (MN-2007), 6.2.2.1 (MN-2007), 6.2.2.2 (MN-2007), 6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.1.3.1 (MN-2007), 6.1.3.2 (MN-2007), 6.1.3.3 (MN-2007), 6.1.1.4 (MN-2007) +4 more</t>
         </is>
       </c>
     </row>
@@ -43635,11 +43835,11 @@
         </is>
       </c>
       <c r="G238" t="n">
-        <v>3</v>
+        <v>16</v>
       </c>
       <c r="H238" s="8" t="inlineStr">
         <is>
-          <t>6.3.5.7 (MN-2022), 6.3.5.8 (MN-2022), 6.3.5.9 (MN-2022)</t>
+          <t>6.2.1.1 (MN-2007), 6.2.2.1 (MN-2007), 6.2.2.2 (MN-2007), 6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.1.3.1 (MN-2007), 6.1.3.2 (MN-2007), 6.1.3.3 (MN-2007), 6.1.1.4 (MN-2007) +6 more</t>
         </is>
       </c>
     </row>
@@ -43669,11 +43869,11 @@
         </is>
       </c>
       <c r="G239" t="n">
-        <v>2</v>
+        <v>18</v>
       </c>
       <c r="H239" s="8" t="inlineStr">
         <is>
-          <t>6.2.3.4 (MN-2022), 6.3.5.7 (MN-2022)</t>
+          <t>6.3.1.1 (MN-2007), 6.3.1.2 (MN-2007), 6.3.2.1 (MN-2007), 6.2.1.1 (MN-2007), 6.2.2.1 (MN-2007), 6.2.2.2 (MN-2007), 6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.1.3.1 (MN-2007) +8 more</t>
         </is>
       </c>
     </row>
@@ -43733,11 +43933,11 @@
         </is>
       </c>
       <c r="G241" t="n">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="H241" s="8" t="inlineStr">
         <is>
-          <t>6.3.5.8 (MN-2022), 6.3.5.9 (MN-2022)</t>
+          <t>6.2.1.1 (MN-2007), 6.2.2.1 (MN-2007), 6.2.2.2 (MN-2007), 6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.1.3.1 (MN-2007), 6.1.3.2 (MN-2007), 6.1.3.3 (MN-2007), 6.1.1.4 (MN-2007) +5 more</t>
         </is>
       </c>
     </row>
@@ -43763,11 +43963,11 @@
       </c>
       <c r="F242" s="8" t="inlineStr"/>
       <c r="G242" t="n">
-        <v>3</v>
+        <v>16</v>
       </c>
       <c r="H242" s="8" t="inlineStr">
         <is>
-          <t>6.3.6.3 (MN-2022), 6.3.6.4 (MN-2022), 6.3.7.1 (MN-2022)</t>
+          <t>6.2.1.1 (MN-2007), 6.2.2.1 (MN-2007), 6.2.2.2 (MN-2007), 6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.1.3.1 (MN-2007), 6.1.3.2 (MN-2007), 6.1.3.3 (MN-2007), 6.1.1.4 (MN-2007) +6 more</t>
         </is>
       </c>
     </row>
@@ -43793,11 +43993,11 @@
       </c>
       <c r="F243" s="8" t="inlineStr"/>
       <c r="G243" t="n">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="H243" s="8" t="inlineStr">
         <is>
-          <t>6.3.6.1 (MN-2022), 6.3.7.1 (MN-2022)</t>
+          <t>6.2.1.1 (MN-2007), 6.2.2.1 (MN-2007), 6.2.2.2 (MN-2007), 6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.1.3.1 (MN-2007), 6.1.3.2 (MN-2007), 6.1.3.3 (MN-2007), 6.1.1.4 (MN-2007) +5 more</t>
         </is>
       </c>
     </row>
@@ -43823,11 +44023,11 @@
       </c>
       <c r="F244" s="8" t="inlineStr"/>
       <c r="G244" t="n">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="H244" s="8" t="inlineStr">
         <is>
-          <t>6.3.6.1 (MN-2022)</t>
+          <t>6.2.1.1 (MN-2007), 6.2.2.1 (MN-2007), 6.2.2.2 (MN-2007), 6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.1.3.1 (MN-2007), 6.1.3.2 (MN-2007), 6.1.3.3 (MN-2007), 6.1.1.4 (MN-2007) +4 more</t>
         </is>
       </c>
     </row>
@@ -43853,11 +44053,11 @@
       </c>
       <c r="F245" s="8" t="inlineStr"/>
       <c r="G245" t="n">
-        <v>6</v>
+        <v>22</v>
       </c>
       <c r="H245" s="8" t="inlineStr">
         <is>
-          <t>6.2.3.3 (MN-2022), 6.2.3.4 (MN-2022), 6.3.5.10 (MN-2022), 6.3.6.3 (MN-2022), 6.3.6.4 (MN-2022), 6.3.7.1 (MN-2022)</t>
+          <t>6.3.1.1 (MN-2007), 6.3.1.2 (MN-2007), 6.3.2.1 (MN-2007), 6.2.1.1 (MN-2007), 6.2.2.1 (MN-2007), 6.2.2.2 (MN-2007), 6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.1.3.1 (MN-2007) +12 more</t>
         </is>
       </c>
     </row>
@@ -43883,11 +44083,11 @@
       </c>
       <c r="F246" s="8" t="inlineStr"/>
       <c r="G246" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H246" s="8" t="inlineStr">
         <is>
-          <t>6.2.4.1 (MN-2022)</t>
+          <t>6.3.1.1 (MN-2007), 6.3.1.2 (MN-2007), 6.3.2.1 (MN-2007), 6.2.4.1 (MN-2022)</t>
         </is>
       </c>
     </row>
@@ -43913,11 +44113,11 @@
       </c>
       <c r="F247" s="8" t="inlineStr"/>
       <c r="G247" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H247" s="8" t="inlineStr">
         <is>
-          <t>6.2.4.2 (MN-2022)</t>
+          <t>6.3.1.1 (MN-2007), 6.3.1.2 (MN-2007), 6.3.2.1 (MN-2007), 6.2.4.2 (MN-2022)</t>
         </is>
       </c>
     </row>
@@ -43943,11 +44143,11 @@
       </c>
       <c r="F248" s="8" t="inlineStr"/>
       <c r="G248" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H248" s="8" t="inlineStr">
         <is>
-          <t>6.2.3.1 (MN-2022), 6.2.3.2 (MN-2022)</t>
+          <t>6.3.1.1 (MN-2007), 6.3.1.2 (MN-2007), 6.3.2.1 (MN-2007), 6.2.3.1 (MN-2022), 6.2.3.2 (MN-2022)</t>
         </is>
       </c>
     </row>
@@ -43973,11 +44173,11 @@
       </c>
       <c r="F249" s="8" t="inlineStr"/>
       <c r="G249" t="n">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="H249" s="8" t="inlineStr">
         <is>
-          <t>6.3.5.11 (MN-2022), 6.3.6.6 (MN-2022)</t>
+          <t>6.2.1.1 (MN-2007), 6.2.2.1 (MN-2007), 6.2.2.2 (MN-2007), 6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.1.3.1 (MN-2007), 6.1.3.2 (MN-2007), 6.1.3.3 (MN-2007), 6.1.1.4 (MN-2007) +5 more</t>
         </is>
       </c>
     </row>
@@ -44177,11 +44377,11 @@
         </is>
       </c>
       <c r="G255" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="H255" s="8" t="inlineStr">
         <is>
-          <t>7.SP.C.5 (CCSS-M), 7.SP.C.6 (CCSS-M), 7.1.2.1 (MN-2022), 7.1.2.2 (MN-2022), 7.SP.6 (CCSS-M), 7.SP.5 (CCSS-M), 7.SP.8c (CCSS-M)</t>
+          <t>7.SP.C.5 (CCSS-M), 7.SP.C.6 (CCSS-M), 7.4.3.1 (MN-2007), 7.4.3.2 (MN-2007), 7.4.1.1 (MN-2007), 7.4.2.1 (MN-2007), 7.1.2.1 (MN-2022), 7.1.2.2 (MN-2022), 7.SP.6 (CCSS-M), 7.SP.5 (CCSS-M) +1 more</t>
         </is>
       </c>
     </row>
@@ -44211,11 +44411,11 @@
         </is>
       </c>
       <c r="G256" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="H256" s="8" t="inlineStr">
         <is>
-          <t>7.SP.C.6 (CCSS-M), 7.1.2.1 (MN-2022), 7.1.2.2 (MN-2022), 7.SP.C.7.B (CCSS-M), 7.SP.7b (CCSS-M), 7.SP.6 (CCSS-M), 7.SP.8c (CCSS-M)</t>
+          <t>7.SP.C.6 (CCSS-M), 7.4.3.1 (MN-2007), 7.4.3.2 (MN-2007), 7.4.1.1 (MN-2007), 7.4.2.1 (MN-2007), 7.1.2.1 (MN-2022), 7.1.2.2 (MN-2022), 7.SP.C.7.B (CCSS-M), 7.SP.7b (CCSS-M), 7.SP.6 (CCSS-M) +1 more</t>
         </is>
       </c>
     </row>
@@ -44381,11 +44581,11 @@
         </is>
       </c>
       <c r="G261" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="H261" s="8" t="inlineStr">
         <is>
-          <t>7.SP.C.8 (CCSS-M), 7.1.2.3 (MN-2022), 7.SP.8a (CCSS-M), 7.SP.8c (CCSS-M)</t>
+          <t>7.SP.C.8 (CCSS-M), 7.4.3.1 (MN-2007), 7.4.3.2 (MN-2007), 7.4.1.1 (MN-2007), 7.4.2.1 (MN-2007), 7.1.2.3 (MN-2022), 7.SP.8a (CCSS-M), 7.SP.8c (CCSS-M)</t>
         </is>
       </c>
     </row>
@@ -44415,11 +44615,11 @@
         </is>
       </c>
       <c r="G262" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="H262" s="8" t="inlineStr">
         <is>
-          <t>7.1.2.3 (MN-2022), 7.SP.C.8.A (CCSS-M), 7.SP.8a (CCSS-M), 7.SP.8c (CCSS-M)</t>
+          <t>7.4.3.1 (MN-2007), 7.4.3.2 (MN-2007), 7.4.1.1 (MN-2007), 7.4.2.1 (MN-2007), 7.1.2.3 (MN-2022), 7.SP.C.8.A (CCSS-M), 7.SP.8a (CCSS-M), 7.SP.8c (CCSS-M)</t>
         </is>
       </c>
     </row>
@@ -44449,11 +44649,11 @@
         </is>
       </c>
       <c r="G263" t="n">
-        <v>6</v>
+        <v>19</v>
       </c>
       <c r="H263" s="8" t="inlineStr">
         <is>
-          <t>7.1.2.1 (MN-2022), 7.1.2.2 (MN-2022), 7.3.5.1 (MN-2022), 7.NS.A.2.D (CCSS-M), 7.NS.2d (CCSS-M), 7.SP.8c (CCSS-M)</t>
+          <t>7.2.3.1 (MN-2007), 7.2.3.2 (MN-2007), 7.1.2.1 (MN-2007), 7.1.2.2 (MN-2007), 7.1.2.3 (MN-2007), 7.2.2.1 (MN-2007), 7.2.2.2 (MN-2007), 7.4.3.1 (MN-2007), 7.4.3.2 (MN-2007), 7.2.1.1 (MN-2007) +9 more</t>
         </is>
       </c>
     </row>
@@ -44485,11 +44685,11 @@
         </is>
       </c>
       <c r="G264" t="n">
-        <v>6</v>
+        <v>19</v>
       </c>
       <c r="H264" s="8" t="inlineStr">
         <is>
-          <t>7.1.2.1 (MN-2022), 7.1.2.2 (MN-2022), 7.3.5.1 (MN-2022), 7.NS.A.2.D (CCSS-M), 7.NS.2d (CCSS-M), 7.SP.8c (CCSS-M)</t>
+          <t>7.2.3.1 (MN-2007), 7.2.3.2 (MN-2007), 7.1.2.1 (MN-2007), 7.1.2.2 (MN-2007), 7.1.2.3 (MN-2007), 7.2.2.1 (MN-2007), 7.2.2.2 (MN-2007), 7.4.3.1 (MN-2007), 7.4.3.2 (MN-2007), 7.2.1.1 (MN-2007) +9 more</t>
         </is>
       </c>
     </row>
@@ -44519,11 +44719,11 @@
         </is>
       </c>
       <c r="G265" t="n">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="H265" s="8" t="inlineStr">
         <is>
-          <t>7.3.5.5 (MN-2022), 7.NS.A.1.D (CCSS-M), 7.RP.2b (CCSS-M), 7.SP.8c (CCSS-M)</t>
+          <t>7.2.3.1 (MN-2007), 7.2.3.2 (MN-2007), 7.1.2.1 (MN-2007), 7.1.2.2 (MN-2007), 7.1.2.3 (MN-2007), 7.2.2.1 (MN-2007), 7.2.2.2 (MN-2007), 7.2.1.1 (MN-2007), 7.2.1.2 (MN-2007), 7.3.5.5 (MN-2022) +3 more</t>
         </is>
       </c>
     </row>
@@ -44553,11 +44753,11 @@
         </is>
       </c>
       <c r="G266" t="n">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="H266" s="8" t="inlineStr">
         <is>
-          <t>7.3.5.2 (MN-2022), 7.3.5.6 (MN-2022), 7.NS.A.1.D (CCSS-M), 7.NS.A.1.A (CCSS-M), 7.NS.A.1.B (CCSS-M), 7.NS.1a (CCSS-M), 7.NS.1b (CCSS-M), 7.NS.1d (CCSS-M), 7.SP.8c (CCSS-M)</t>
+          <t>7.2.3.1 (MN-2007), 7.2.3.2 (MN-2007), 7.1.2.1 (MN-2007), 7.1.2.2 (MN-2007), 7.1.2.3 (MN-2007), 7.2.2.1 (MN-2007), 7.2.2.2 (MN-2007), 7.2.1.1 (MN-2007), 7.2.1.2 (MN-2007), 7.3.5.2 (MN-2022) +8 more</t>
         </is>
       </c>
     </row>
@@ -44587,11 +44787,11 @@
         </is>
       </c>
       <c r="G267" t="n">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="H267" s="8" t="inlineStr">
         <is>
-          <t>7.3.5.2 (MN-2022), 7.3.5.5 (MN-2022), 7.3.5.6 (MN-2022), 7.NS.A.1.D (CCSS-M), 7.NS.A.1.A (CCSS-M), 7.NS.A.1.B (CCSS-M), 7.NS.1a (CCSS-M), 7.NS.1b (CCSS-M), 7.NS.1d (CCSS-M), 7.SP.8c (CCSS-M)</t>
+          <t>7.2.3.1 (MN-2007), 7.2.3.2 (MN-2007), 7.1.2.1 (MN-2007), 7.1.2.2 (MN-2007), 7.1.2.3 (MN-2007), 7.2.2.1 (MN-2007), 7.2.2.2 (MN-2007), 7.2.1.1 (MN-2007), 7.2.1.2 (MN-2007), 7.3.5.2 (MN-2022) +9 more</t>
         </is>
       </c>
     </row>
@@ -44621,11 +44821,11 @@
         </is>
       </c>
       <c r="G268" t="n">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="H268" s="8" t="inlineStr">
         <is>
-          <t>7.3.5.2 (MN-2022), 7.NS.A.2.A (CCSS-M), 7.NS.2a (CCSS-M), 7.SP.8c (CCSS-M)</t>
+          <t>7.2.3.1 (MN-2007), 7.2.3.2 (MN-2007), 7.1.2.1 (MN-2007), 7.1.2.2 (MN-2007), 7.1.2.3 (MN-2007), 7.2.2.1 (MN-2007), 7.2.2.2 (MN-2007), 7.2.1.1 (MN-2007), 7.2.1.2 (MN-2007), 7.3.5.2 (MN-2022) +3 more</t>
         </is>
       </c>
     </row>
@@ -44792,11 +44992,11 @@
         </is>
       </c>
       <c r="G273" t="n">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="H273" s="8" t="inlineStr">
         <is>
-          <t>7.3.5.6 (MN-2022), 7.NS.A.2.D (CCSS-M), 7.RP.2b (CCSS-M), 7.NS.1d (CCSS-M)</t>
+          <t>7.2.3.1 (MN-2007), 7.2.3.2 (MN-2007), 7.1.2.1 (MN-2007), 7.1.2.2 (MN-2007), 7.1.2.3 (MN-2007), 7.2.2.1 (MN-2007), 7.2.2.2 (MN-2007), 7.2.1.1 (MN-2007), 7.2.1.2 (MN-2007), 7.3.5.6 (MN-2022) +3 more</t>
         </is>
       </c>
     </row>
@@ -44826,11 +45026,11 @@
         </is>
       </c>
       <c r="G274" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="H274" s="8" t="inlineStr">
         <is>
-          <t>7.NS.A.3 (CCSS-M), 7.3.6.3 (MN-2022), 7.RP.2b (CCSS-M)</t>
+          <t>7.2.3.1 (MN-2007), 7.2.3.2 (MN-2007), 7.NS.A.3 (CCSS-M), 7.1.2.1 (MN-2007), 7.1.2.2 (MN-2007), 7.1.2.3 (MN-2007), 7.2.2.1 (MN-2007), 7.2.2.2 (MN-2007), 7.2.1.1 (MN-2007), 7.2.1.2 (MN-2007) +2 more</t>
         </is>
       </c>
     </row>
@@ -44860,11 +45060,11 @@
         </is>
       </c>
       <c r="G275" t="n">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="H275" s="8" t="inlineStr">
         <is>
-          <t>7.3.5.4 (MN-2022), 7.3.5.5 (MN-2022), 7.3.6.3 (MN-2022), 7.NS.A.1.D (CCSS-M), 7.NS.A.1.C (CCSS-M), 7.RP.2b (CCSS-M), 7.NS.1c (CCSS-M), 7.NS.1d (CCSS-M)</t>
+          <t>7.2.3.1 (MN-2007), 7.2.3.2 (MN-2007), 7.1.2.1 (MN-2007), 7.1.2.2 (MN-2007), 7.1.2.3 (MN-2007), 7.2.2.1 (MN-2007), 7.2.2.2 (MN-2007), 7.2.1.1 (MN-2007), 7.2.1.2 (MN-2007), 7.3.5.4 (MN-2022) +7 more</t>
         </is>
       </c>
     </row>
@@ -44928,11 +45128,11 @@
         </is>
       </c>
       <c r="G277" t="n">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="H277" s="8" t="inlineStr">
         <is>
-          <t>7.3.5.4 (MN-2022), 7.NS.A.2.A (CCSS-M), 7.NS.A.2.C (CCSS-M), 7.RP.2b (CCSS-M), 7.NS.2a (CCSS-M), 7.NS.2b (CCSS-M), 7.NS.2c (CCSS-M)</t>
+          <t>7.2.3.1 (MN-2007), 7.2.3.2 (MN-2007), 7.1.2.1 (MN-2007), 7.1.2.2 (MN-2007), 7.1.2.3 (MN-2007), 7.2.2.1 (MN-2007), 7.2.2.2 (MN-2007), 7.2.1.1 (MN-2007), 7.2.1.2 (MN-2007), 7.3.5.4 (MN-2022) +6 more</t>
         </is>
       </c>
     </row>
@@ -44996,11 +45196,11 @@
         </is>
       </c>
       <c r="G279" t="n">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="H279" s="8" t="inlineStr">
         <is>
-          <t>7.NS.A.3 (CCSS-M), 7.3.5.5 (MN-2022), 7.3.6.5 (MN-2022), 7.NS.A.2.C (CCSS-M), 7.RP.2b (CCSS-M), 7.NS.3 (CCSS-M)</t>
+          <t>7.2.3.1 (MN-2007), 7.2.3.2 (MN-2007), 7.NS.A.3 (CCSS-M), 7.1.2.1 (MN-2007), 7.1.2.2 (MN-2007), 7.1.2.3 (MN-2007), 7.2.2.1 (MN-2007), 7.2.2.2 (MN-2007), 7.2.1.1 (MN-2007), 7.2.1.2 (MN-2007) +5 more</t>
         </is>
       </c>
     </row>
@@ -45030,11 +45230,11 @@
         </is>
       </c>
       <c r="G280" t="n">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="H280" s="8" t="inlineStr">
         <is>
-          <t>7.NS.A.3 (CCSS-M), 7.3.6.5 (MN-2022), 7.NS.A.2.C (CCSS-M), 7.RP.2b (CCSS-M), 7.NS.2b (CCSS-M), 7.NS.3 (CCSS-M)</t>
+          <t>7.2.3.1 (MN-2007), 7.2.3.2 (MN-2007), 7.NS.A.3 (CCSS-M), 7.1.2.1 (MN-2007), 7.1.2.2 (MN-2007), 7.1.2.3 (MN-2007), 7.2.2.1 (MN-2007), 7.2.2.2 (MN-2007), 7.2.1.1 (MN-2007), 7.2.1.2 (MN-2007) +5 more</t>
         </is>
       </c>
     </row>
@@ -45098,11 +45298,11 @@
         </is>
       </c>
       <c r="G282" t="n">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="H282" s="8" t="inlineStr">
         <is>
-          <t>7.NS.A.3 (CCSS-M), 7.3.5.6 (MN-2022), 7.3.6.5 (MN-2022), 7.NS.A.1.D (CCSS-M), 7.NS.A.2.C (CCSS-M), 7.RP.2b (CCSS-M), 7.NS.1d (CCSS-M), 7.NS.2c (CCSS-M), 7.NS.3 (CCSS-M)</t>
+          <t>7.2.3.1 (MN-2007), 7.2.3.2 (MN-2007), 7.NS.A.3 (CCSS-M), 7.1.2.1 (MN-2007), 7.1.2.2 (MN-2007), 7.1.2.3 (MN-2007), 7.2.2.1 (MN-2007), 7.2.2.2 (MN-2007), 7.2.1.1 (MN-2007), 7.2.1.2 (MN-2007) +8 more</t>
         </is>
       </c>
     </row>
@@ -45132,11 +45332,11 @@
         </is>
       </c>
       <c r="G283" t="n">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="H283" s="8" t="inlineStr">
         <is>
-          <t>7.G.A.1 (CCSS-M), 7.2.4.2 (MN-2022), 7.2.4.4 (MN-2022), 7.3.5.7 (MN-2022), 7.RP.2b (CCSS-M), 7.G.1 (CCSS-M)</t>
+          <t>7.3.2.2 (MN-2007), 7.3.2.3 (MN-2007), 7.3.2.1 (MN-2007), 7.2.3.1 (MN-2007), 7.2.3.2 (MN-2007), 7.1.2.1 (MN-2007), 7.1.2.2 (MN-2007), 7.1.2.3 (MN-2007), 7.2.2.1 (MN-2007), 7.2.2.2 (MN-2007) +10 more</t>
         </is>
       </c>
     </row>
@@ -45166,11 +45366,11 @@
         </is>
       </c>
       <c r="G284" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="H284" s="8" t="inlineStr">
         <is>
-          <t>7.G.A.1 (CCSS-M), 7.2.4.2 (MN-2022), 7.2.4.4 (MN-2022), 7.RP.2b (CCSS-M), 7.G.1 (CCSS-M)</t>
+          <t>7.3.2.2 (MN-2007), 7.3.2.3 (MN-2007), 7.3.2.1 (MN-2007), 7.G.A.1 (CCSS-M), 7.3.1.1 (MN-2007), 7.3.1.2 (MN-2007), 7.2.4.2 (MN-2022), 7.2.4.4 (MN-2022), 7.RP.2b (CCSS-M), 7.G.1 (CCSS-M)</t>
         </is>
       </c>
     </row>
@@ -45200,11 +45400,11 @@
         </is>
       </c>
       <c r="G285" t="n">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="H285" s="8" t="inlineStr">
         <is>
-          <t>7.3.7.2 (MN-2022), 7.RP.A.2.A (CCSS-M), 7.RP.2a (CCSS-M), 7.RP.2b (CCSS-M)</t>
+          <t>7.2.3.1 (MN-2007), 7.2.3.2 (MN-2007), 7.1.2.1 (MN-2007), 7.1.2.2 (MN-2007), 7.1.2.3 (MN-2007), 7.2.2.1 (MN-2007), 7.2.2.2 (MN-2007), 7.2.1.1 (MN-2007), 7.2.1.2 (MN-2007), 7.3.7.2 (MN-2022) +3 more</t>
         </is>
       </c>
     </row>
@@ -45234,11 +45434,11 @@
         </is>
       </c>
       <c r="G286" t="n">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="H286" s="8" t="inlineStr">
         <is>
-          <t>7.3.7.1 (MN-2022), 7.3.7.3 (MN-2022), 7.RP.A.2.A (CCSS-M), 7.RP.A.2.D (CCSS-M), 7.RP.2b (CCSS-M), 7.RP.2d (CCSS-M)</t>
+          <t>7.2.3.1 (MN-2007), 7.2.3.2 (MN-2007), 7.1.2.1 (MN-2007), 7.1.2.2 (MN-2007), 7.1.2.3 (MN-2007), 7.2.2.1 (MN-2007), 7.2.2.2 (MN-2007), 7.2.1.1 (MN-2007), 7.2.1.2 (MN-2007), 7.3.7.1 (MN-2022) +5 more</t>
         </is>
       </c>
     </row>
@@ -45268,11 +45468,11 @@
         </is>
       </c>
       <c r="G287" t="n">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="H287" s="8" t="inlineStr">
         <is>
-          <t>7.RP.A.1 (CCSS-M), 7.3.5.7 (MN-2022), 7.RP.A.2.A (CCSS-M), 7.RP.A.2.D (CCSS-M), 7.RP.A.2.B (CCSS-M), 7.RP.A.2.C (CCSS-M), 7.RP.1 (CCSS-M), 7.RP.2b (CCSS-M), 7.RP.2c (CCSS-M)</t>
+          <t>7.2.3.1 (MN-2007), 7.2.3.2 (MN-2007), 7.1.2.1 (MN-2007), 7.1.2.2 (MN-2007), 7.1.2.3 (MN-2007), 7.2.2.1 (MN-2007), 7.2.2.2 (MN-2007), 7.RP.A.1 (CCSS-M), 7.2.1.1 (MN-2007), 7.2.1.2 (MN-2007) +8 more</t>
         </is>
       </c>
     </row>
@@ -45302,11 +45502,11 @@
         </is>
       </c>
       <c r="G288" t="n">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="H288" s="8" t="inlineStr">
         <is>
-          <t>7.3.7.1 (MN-2022), 7.3.7.2 (MN-2022), 7.3.7.3 (MN-2022), 7.RP.A.2.A (CCSS-M), 7.RP.A.2.D (CCSS-M), 7.RP.A.2.B (CCSS-M), 7.RP.A.2.C (CCSS-M), 7.RP.2a (CCSS-M), 7.RP.2b (CCSS-M), 7.RP.2c (CCSS-M) +1 more</t>
+          <t>7.2.3.1 (MN-2007), 7.2.3.2 (MN-2007), 7.1.2.1 (MN-2007), 7.1.2.2 (MN-2007), 7.1.2.3 (MN-2007), 7.2.2.1 (MN-2007), 7.2.2.2 (MN-2007), 7.2.1.1 (MN-2007), 7.2.1.2 (MN-2007), 7.3.7.1 (MN-2022) +10 more</t>
         </is>
       </c>
     </row>
@@ -45336,11 +45536,11 @@
         </is>
       </c>
       <c r="G289" t="n">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="H289" s="8" t="inlineStr">
         <is>
-          <t>7.EE.A.1 (CCSS-M), 7.3.6.1 (MN-2022), 7.RP.2b (CCSS-M), 7.EE.1 (CCSS-M)</t>
+          <t>7.EE.A.1 (CCSS-M), 7.2.3.1 (MN-2007), 7.2.3.2 (MN-2007), 7.1.2.1 (MN-2007), 7.1.2.2 (MN-2007), 7.1.2.3 (MN-2007), 7.2.2.1 (MN-2007), 7.2.2.2 (MN-2007), 7.2.1.1 (MN-2007), 7.2.1.2 (MN-2007) +3 more</t>
         </is>
       </c>
     </row>
@@ -45404,11 +45604,11 @@
         </is>
       </c>
       <c r="G291" t="n">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="H291" s="8" t="inlineStr">
         <is>
-          <t>7.EE.A.1 (CCSS-M), 7.3.6.1 (MN-2022), 7.RP.2b (CCSS-M), 7.EE.1 (CCSS-M)</t>
+          <t>7.EE.A.1 (CCSS-M), 7.2.3.1 (MN-2007), 7.2.3.2 (MN-2007), 7.1.2.1 (MN-2007), 7.1.2.2 (MN-2007), 7.1.2.3 (MN-2007), 7.2.2.1 (MN-2007), 7.2.2.2 (MN-2007), 7.2.1.1 (MN-2007), 7.2.1.2 (MN-2007) +3 more</t>
         </is>
       </c>
     </row>
@@ -45434,11 +45634,11 @@
       </c>
       <c r="F292" s="8" t="inlineStr"/>
       <c r="G292" t="n">
-        <v>3</v>
+        <v>17</v>
       </c>
       <c r="H292" s="8" t="inlineStr">
         <is>
-          <t>7.2.4.3 (MN-2022), 7.2.4.4 (MN-2022), 7.3.5.7 (MN-2022)</t>
+          <t>7.3.2.2 (MN-2007), 7.3.2.3 (MN-2007), 7.3.2.1 (MN-2007), 7.2.3.1 (MN-2007), 7.2.3.2 (MN-2007), 7.1.2.1 (MN-2007), 7.1.2.2 (MN-2007), 7.1.2.3 (MN-2007), 7.2.2.1 (MN-2007), 7.2.2.2 (MN-2007) +7 more</t>
         </is>
       </c>
     </row>
@@ -45468,11 +45668,11 @@
         </is>
       </c>
       <c r="G293" t="n">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="H293" s="8" t="inlineStr">
         <is>
-          <t>7.3.5.5 (MN-2022), 7.3.6.4 (MN-2022), 7.RP.3 (CCSS-M), 7.RP.2b (CCSS-M)</t>
+          <t>7.2.3.1 (MN-2007), 7.2.3.2 (MN-2007), 7.1.2.1 (MN-2007), 7.1.2.2 (MN-2007), 7.1.2.3 (MN-2007), 7.2.2.1 (MN-2007), 7.2.2.2 (MN-2007), 7.2.1.1 (MN-2007), 7.2.1.2 (MN-2007), 7.3.5.5 (MN-2022) +3 more</t>
         </is>
       </c>
     </row>
@@ -45502,11 +45702,11 @@
         </is>
       </c>
       <c r="G294" t="n">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="H294" s="8" t="inlineStr">
         <is>
-          <t>7.3.5.5 (MN-2022), 7.3.6.4 (MN-2022), 7.RP.3 (CCSS-M), 7.RP.2b (CCSS-M)</t>
+          <t>7.2.3.1 (MN-2007), 7.2.3.2 (MN-2007), 7.1.2.1 (MN-2007), 7.1.2.2 (MN-2007), 7.1.2.3 (MN-2007), 7.2.2.1 (MN-2007), 7.2.2.2 (MN-2007), 7.2.1.1 (MN-2007), 7.2.1.2 (MN-2007), 7.3.5.5 (MN-2022) +3 more</t>
         </is>
       </c>
     </row>
@@ -45570,11 +45770,11 @@
         </is>
       </c>
       <c r="G296" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="H296" s="8" t="inlineStr">
         <is>
-          <t>7.1.2.5 (MN-2022), 7.1.2.6 (MN-2022), 7.SP.7b (CCSS-M), 7.SP.7c (CCSS-M), 7.RP.2b (CCSS-M), 7.SP.8c (CCSS-M)</t>
+          <t>7.4.3.1 (MN-2007), 7.4.3.2 (MN-2007), 7.4.1.1 (MN-2007), 7.4.2.1 (MN-2007), 7.1.2.5 (MN-2022), 7.1.2.6 (MN-2022), 7.SP.7b (CCSS-M), 7.SP.7c (CCSS-M), 7.RP.2b (CCSS-M), 7.SP.8c (CCSS-M)</t>
         </is>
       </c>
     </row>
@@ -45604,11 +45804,11 @@
         </is>
       </c>
       <c r="G297" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="H297" s="8" t="inlineStr">
         <is>
-          <t>7.1.2.3 (MN-2022), 7.SP.6 (CCSS-M), 7.RP.2b (CCSS-M)</t>
+          <t>7.4.3.1 (MN-2007), 7.4.3.2 (MN-2007), 7.4.1.1 (MN-2007), 7.4.2.1 (MN-2007), 7.1.2.3 (MN-2022), 7.SP.6 (CCSS-M), 7.RP.2b (CCSS-M)</t>
         </is>
       </c>
     </row>
@@ -45638,11 +45838,11 @@
         </is>
       </c>
       <c r="G298" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="H298" s="8" t="inlineStr">
         <is>
-          <t>7.1.2.4 (MN-2022), 7.1.2.6 (MN-2022), 7.SP.8b (CCSS-M), 7.RP.2b (CCSS-M)</t>
+          <t>7.4.3.1 (MN-2007), 7.4.3.2 (MN-2007), 7.4.1.1 (MN-2007), 7.4.2.1 (MN-2007), 7.1.2.4 (MN-2022), 7.1.2.6 (MN-2022), 7.SP.8b (CCSS-M), 7.RP.2b (CCSS-M)</t>
         </is>
       </c>
     </row>
@@ -45672,11 +45872,11 @@
         </is>
       </c>
       <c r="G299" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="H299" s="8" t="inlineStr">
         <is>
-          <t>7.1.2.4 (MN-2022), 7.1.2.6 (MN-2022), 7.Sp.8a (CCSS-M), 7.SP.8a (CCSS-M), 7.RP.2b (CCSS-M)</t>
+          <t>7.4.3.1 (MN-2007), 7.4.3.2 (MN-2007), 7.4.1.1 (MN-2007), 7.4.2.1 (MN-2007), 7.1.2.4 (MN-2022), 7.1.2.6 (MN-2022), 7.Sp.8a (CCSS-M), 7.SP.8a (CCSS-M), 7.RP.2b (CCSS-M)</t>
         </is>
       </c>
     </row>
@@ -45706,11 +45906,11 @@
         </is>
       </c>
       <c r="G300" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="H300" s="8" t="inlineStr">
         <is>
-          <t>7.1.2.3 (MN-2022), 7.SP.8b (CCSS-M), 7.SP.8a (CCSS-M), 7.RP.2b (CCSS-M)</t>
+          <t>7.4.3.1 (MN-2007), 7.4.3.2 (MN-2007), 7.4.1.1 (MN-2007), 7.4.2.1 (MN-2007), 7.1.2.3 (MN-2022), 7.SP.8b (CCSS-M), 7.SP.8a (CCSS-M), 7.RP.2b (CCSS-M)</t>
         </is>
       </c>
     </row>
@@ -45910,11 +46110,11 @@
         </is>
       </c>
       <c r="G306" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="H306" s="8" t="inlineStr">
         <is>
-          <t>7.2.4.1 (MN-2022), 7.EE.4a (CCSS-M), 7.EE.4b (CCSS-M), 7.RP.2b (CCSS-M)</t>
+          <t>7.3.2.2 (MN-2007), 7.3.2.3 (MN-2007), 7.3.2.1 (MN-2007), 7.3.1.1 (MN-2007), 7.3.1.2 (MN-2007), 7.2.4.1 (MN-2022), 7.EE.4a (CCSS-M), 7.EE.4b (CCSS-M), 7.RP.2b (CCSS-M)</t>
         </is>
       </c>
     </row>
@@ -45978,11 +46178,11 @@
         </is>
       </c>
       <c r="G308" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="H308" s="8" t="inlineStr">
         <is>
-          <t>7.2.4.1 (MN-2022), 7.EE.4a (CCSS-M), 7.EE.4b (CCSS-M), 7.RP.2b (CCSS-M)</t>
+          <t>7.3.2.2 (MN-2007), 7.3.2.3 (MN-2007), 7.3.2.1 (MN-2007), 7.3.1.1 (MN-2007), 7.3.1.2 (MN-2007), 7.2.4.1 (MN-2022), 7.EE.4a (CCSS-M), 7.EE.4b (CCSS-M), 7.RP.2b (CCSS-M)</t>
         </is>
       </c>
     </row>
@@ -46114,11 +46314,11 @@
         </is>
       </c>
       <c r="G312" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="H312" s="8" t="inlineStr">
         <is>
-          <t>7.2.4.1 (MN-2022), 7.EE.3 (CCSS-M), 7.EE.4a (CCSS-M), 7.RP.2b (CCSS-M)</t>
+          <t>7.3.2.2 (MN-2007), 7.3.2.3 (MN-2007), 7.3.2.1 (MN-2007), 7.3.1.1 (MN-2007), 7.3.1.2 (MN-2007), 7.2.4.1 (MN-2022), 7.EE.3 (CCSS-M), 7.EE.4a (CCSS-M), 7.RP.2b (CCSS-M)</t>
         </is>
       </c>
     </row>
@@ -46284,11 +46484,11 @@
         </is>
       </c>
       <c r="G317" t="n">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="H317" s="8" t="inlineStr">
         <is>
-          <t>7.3.5.3 (MN-2022), 7.RP.3 (CCSS-M), see ebook (CCSS-M), 7.RP.2b (CCSS-M), 7.RP.2c (CCSS-M), 7.RP.2d (CCSS-M)</t>
+          <t>7.2.3.1 (MN-2007), 7.2.3.2 (MN-2007), 7.1.2.1 (MN-2007), 7.1.2.2 (MN-2007), 7.1.2.3 (MN-2007), 7.2.2.1 (MN-2007), 7.2.2.2 (MN-2007), 7.2.1.1 (MN-2007), 7.2.1.2 (MN-2007), 7.3.5.3 (MN-2022) +5 more</t>
         </is>
       </c>
     </row>
@@ -46386,11 +46586,11 @@
         </is>
       </c>
       <c r="G320" t="n">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="H320" s="8" t="inlineStr">
         <is>
-          <t>7.3.5.3 (MN-2022), 7.3.6.2 (MN-2022), see ebook (CCSS-M), 7.RP.2b (CCSS-M), 7.NS.3 (CCSS-M)</t>
+          <t>7.2.3.1 (MN-2007), 7.2.3.2 (MN-2007), 7.1.2.1 (MN-2007), 7.1.2.2 (MN-2007), 7.1.2.3 (MN-2007), 7.2.2.1 (MN-2007), 7.2.2.2 (MN-2007), 7.2.1.1 (MN-2007), 7.2.1.2 (MN-2007), 7.3.5.3 (MN-2022) +4 more</t>
         </is>
       </c>
     </row>
@@ -46556,11 +46756,11 @@
         </is>
       </c>
       <c r="G325" t="n">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="H325" s="8" t="inlineStr">
         <is>
-          <t>7.3.6.2 (MN-2022), 7.RP.3 (CCSS-M), see ebook (CCSS-M), 7.RP.2b (CCSS-M)</t>
+          <t>7.2.3.1 (MN-2007), 7.2.3.2 (MN-2007), 7.1.2.1 (MN-2007), 7.1.2.2 (MN-2007), 7.1.2.3 (MN-2007), 7.2.2.1 (MN-2007), 7.2.2.2 (MN-2007), 7.2.1.1 (MN-2007), 7.2.1.2 (MN-2007), 7.3.6.2 (MN-2022) +3 more</t>
         </is>
       </c>
     </row>
@@ -46624,11 +46824,11 @@
         </is>
       </c>
       <c r="G327" t="n">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="H327" s="8" t="inlineStr">
         <is>
-          <t>7.3.6.2 (MN-2022), 7.3.6.4 (MN-2022), 7.3.6.5 (MN-2022), see ebook (CCSS-M), 7.RP.2b (CCSS-M), 7.SP.3 (CCSS-M), 7.2.1 (CCSS-M)</t>
+          <t>7.2.3.1 (MN-2007), 7.2.3.2 (MN-2007), 7.1.2.1 (MN-2007), 7.1.2.2 (MN-2007), 7.1.2.3 (MN-2007), 7.2.2.1 (MN-2007), 7.2.2.2 (MN-2007), 7.2.1.1 (MN-2007), 7.2.1.2 (MN-2007), 7.3.6.2 (MN-2022) +6 more</t>
         </is>
       </c>
     </row>
@@ -46692,11 +46892,11 @@
         </is>
       </c>
       <c r="G329" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="H329" s="8" t="inlineStr">
         <is>
-          <t>7.1.1.1 (MN-2022), 7.1.1.2 (MN-2022), 7.1.1.3 (MN-2022), 7.1.1.6 (MN-2022), see ebook (CCSS-M), 7.RP.2b (CCSS-M), 7.SP.1 (CCSS-M)</t>
+          <t>7.4.3.1 (MN-2007), 7.4.3.2 (MN-2007), 7.4.1.1 (MN-2007), 7.4.2.1 (MN-2007), 7.1.1.1 (MN-2022), 7.1.1.2 (MN-2022), 7.1.1.3 (MN-2022), 7.1.1.6 (MN-2022), see ebook (CCSS-M), 7.RP.2b (CCSS-M) +1 more</t>
         </is>
       </c>
     </row>
@@ -46726,11 +46926,11 @@
         </is>
       </c>
       <c r="G330" t="n">
-        <v>8</v>
+        <v>21</v>
       </c>
       <c r="H330" s="8" t="inlineStr">
         <is>
-          <t>7.1.1.2 (MN-2022), 7.1.1.3 (MN-2022), 7.1.1.6 (MN-2022), 7.3.6.4 (MN-2022), see ebook (CCSS-M), 7.RP.2b (CCSS-M), 7.SP.2 (CCSS-M), 7.SP.4 (CCSS-M)</t>
+          <t>7.2.3.1 (MN-2007), 7.2.3.2 (MN-2007), 7.1.2.1 (MN-2007), 7.1.2.2 (MN-2007), 7.1.2.3 (MN-2007), 7.2.2.1 (MN-2007), 7.2.2.2 (MN-2007), 7.4.3.1 (MN-2007), 7.4.3.2 (MN-2007), 7.2.1.1 (MN-2007) +11 more</t>
         </is>
       </c>
     </row>
@@ -46998,11 +47198,11 @@
         </is>
       </c>
       <c r="G338" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="H338" s="8" t="inlineStr">
         <is>
-          <t>7.1.1.1 (MN-2022), 7.1.1.2 (MN-2022), 7.1.1.3 (MN-2022), see ebook (CCSS-M), 7.RP.2b (CCSS-M)</t>
+          <t>7.4.3.1 (MN-2007), 7.4.3.2 (MN-2007), 7.4.1.1 (MN-2007), 7.4.2.1 (MN-2007), 7.1.1.1 (MN-2022), 7.1.1.2 (MN-2022), 7.1.1.3 (MN-2022), see ebook (CCSS-M), 7.RP.2b (CCSS-M)</t>
         </is>
       </c>
     </row>
@@ -47130,11 +47330,11 @@
       </c>
       <c r="F342" s="8" t="inlineStr"/>
       <c r="G342" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="H342" s="8" t="inlineStr">
         <is>
-          <t>7.1.1.4 (MN-2022), 7.1.1.5 (MN-2022), see ebook (CCSS-M)</t>
+          <t>7.4.3.1 (MN-2007), 7.4.3.2 (MN-2007), 7.4.1.1 (MN-2007), 7.4.2.1 (MN-2007), 7.1.1.4 (MN-2022), 7.1.1.5 (MN-2022), see ebook (CCSS-M)</t>
         </is>
       </c>
     </row>
@@ -47212,11 +47412,11 @@
       </c>
       <c r="F345" s="8" t="inlineStr"/>
       <c r="G345" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="H345" s="8" t="inlineStr">
         <is>
-          <t>7.1.1.5 (MN-2022)</t>
+          <t>7.4.3.1 (MN-2007), 7.4.3.2 (MN-2007), 7.4.1.1 (MN-2007), 7.4.2.1 (MN-2007), 7.1.1.5 (MN-2022)</t>
         </is>
       </c>
     </row>
@@ -47242,11 +47442,11 @@
       </c>
       <c r="F346" s="8" t="inlineStr"/>
       <c r="G346" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="H346" s="8" t="inlineStr">
         <is>
-          <t>7.2.3.1 (MN-2022), 7.2.3.2 (MN-2022), 7.2.3.3 (MN-2022), 7.2.3.4 (MN-2022)</t>
+          <t>7.3.2.2 (MN-2007), 7.3.2.3 (MN-2007), 7.3.2.1 (MN-2007), 7.3.1.1 (MN-2007), 7.3.1.2 (MN-2007), 7.2.3.1 (MN-2022), 7.2.3.2 (MN-2022), 7.2.3.3 (MN-2022), 7.2.3.4 (MN-2022)</t>
         </is>
       </c>
     </row>
@@ -47272,11 +47472,11 @@
       </c>
       <c r="F347" s="8" t="inlineStr"/>
       <c r="G347" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="H347" s="8" t="inlineStr">
         <is>
-          <t>7.2.3.4 (MN-2022)</t>
+          <t>7.3.2.2 (MN-2007), 7.3.2.3 (MN-2007), 7.3.2.1 (MN-2007), 7.3.1.1 (MN-2007), 7.3.1.2 (MN-2007), 7.2.3.4 (MN-2022)</t>
         </is>
       </c>
     </row>
@@ -47302,11 +47502,11 @@
       </c>
       <c r="F348" s="8" t="inlineStr"/>
       <c r="G348" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="H348" s="8" t="inlineStr">
         <is>
-          <t>7.1.1.2 (MN-2022), 7.1.1.3 (MN-2022), 7.1.1.6 (MN-2022)</t>
+          <t>7.4.3.1 (MN-2007), 7.4.3.2 (MN-2007), 7.4.1.1 (MN-2007), 7.4.2.1 (MN-2007), 7.1.1.2 (MN-2022), 7.1.1.3 (MN-2022), 7.1.1.6 (MN-2022)</t>
         </is>
       </c>
     </row>
@@ -47436,11 +47636,11 @@
         </is>
       </c>
       <c r="G352" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H352" s="8" t="inlineStr">
         <is>
-          <t>8.SP.A.1 (CCSS-M), 8.SP.A.2 (CCSS-M), 8.1.1.1 (MN-2022), 8.1.1.5 (MN-2022), 8.1.1.6 (MN-2022), 8.SP.2 (CCSS-M)</t>
+          <t>8.SP.A.1 (CCSS-M), 8.SP.A.2 (CCSS-M), 8.4.1.1 (MN-2007), 8.4.1.2 (MN-2007), 8.1.1.1 (MN-2022), 8.1.1.5 (MN-2022), 8.1.1.6 (MN-2022), 8.SP.2 (CCSS-M)</t>
         </is>
       </c>
     </row>
@@ -47575,11 +47775,11 @@
         </is>
       </c>
       <c r="G356" t="n">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="H356" s="8" t="inlineStr">
         <is>
-          <t>7.EE.A.1 (CCSS-M), 8.3.6.1 (MN-2022), 8.EE.C.7.B (CCSS-M), 8.EE.C.7.A (CCSS-M), 8.EE.7a (CCSS-M)</t>
+          <t>7.EE.A.1 (CCSS-M), 8.2.2.1 (MN-2007), 8.2.2.2 (MN-2007), 8.2.1.1 (MN-2007), 8.2.1.2 (MN-2007), 8.2.3.1 (MN-2007), 8.1.1.1 (MN-2007), 8.1.1.2 (MN-2007), 8.1.2.1 (MN-2007), 8.2.3.2 (MN-2007) +4 more</t>
         </is>
       </c>
     </row>
@@ -47644,11 +47844,11 @@
         </is>
       </c>
       <c r="G358" t="n">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="H358" s="8" t="inlineStr">
         <is>
-          <t>8.3.6.2 (MN-2022), 8.EE.C.7.B (CCSS-M), 8.EE.C.7.A (CCSS-M), 7.EE.A.1.A (CCSS-M), 7.EE.A.1.B (CCSS-M), 8.EE.7a (CCSS-M)</t>
+          <t>8.2.2.1 (MN-2007), 8.2.2.2 (MN-2007), 8.2.1.1 (MN-2007), 8.2.1.2 (MN-2007), 8.2.3.1 (MN-2007), 8.1.1.1 (MN-2007), 8.1.1.2 (MN-2007), 8.1.2.1 (MN-2007), 8.2.3.2 (MN-2007), 8.3.6.2 (MN-2022) +5 more</t>
         </is>
       </c>
     </row>
@@ -47679,11 +47879,11 @@
         </is>
       </c>
       <c r="G359" t="n">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="H359" s="8" t="inlineStr">
         <is>
-          <t>8.3.6.1 (MN-2022), 8.EE.C.7.B (CCSS-M), 8.EE.C.7.A (CCSS-M), 7.EE.B.4.B (CCSS-M), 8.EE.7a (CCSS-M)</t>
+          <t>8.2.2.1 (MN-2007), 8.2.2.2 (MN-2007), 8.2.1.1 (MN-2007), 8.2.1.2 (MN-2007), 8.2.3.1 (MN-2007), 8.1.1.1 (MN-2007), 8.1.1.2 (MN-2007), 8.1.2.1 (MN-2007), 8.2.3.2 (MN-2007), 8.3.6.1 (MN-2022) +4 more</t>
         </is>
       </c>
     </row>
@@ -47749,11 +47949,11 @@
         </is>
       </c>
       <c r="G361" t="n">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="H361" s="8" t="inlineStr">
         <is>
-          <t>8.3.6.1 (MN-2022), 8.EE.C.7.B (CCSS-M), 8.EE.C.7.A (CCSS-M), 7.EE.B.4.B (CCSS-M), 8.EE.7a (CCSS-M)</t>
+          <t>8.2.2.1 (MN-2007), 8.2.2.2 (MN-2007), 8.2.1.1 (MN-2007), 8.2.1.2 (MN-2007), 8.2.3.1 (MN-2007), 8.1.1.1 (MN-2007), 8.1.1.2 (MN-2007), 8.1.2.1 (MN-2007), 8.2.3.2 (MN-2007), 8.3.6.1 (MN-2022) +4 more</t>
         </is>
       </c>
     </row>
@@ -47783,11 +47983,11 @@
         </is>
       </c>
       <c r="G362" t="n">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="H362" s="8" t="inlineStr">
         <is>
-          <t>8.3.6.3 (MN-2022), 8.EE.C.7.B (CCSS-M), 8.EE.C.7.A (CCSS-M), 8.EE.7a (CCSS-M), 8.EE.7b (CCSS-M)</t>
+          <t>8.2.2.1 (MN-2007), 8.2.2.2 (MN-2007), 8.2.1.1 (MN-2007), 8.2.1.2 (MN-2007), 8.2.3.1 (MN-2007), 8.1.1.1 (MN-2007), 8.1.1.2 (MN-2007), 8.1.2.1 (MN-2007), 8.2.3.2 (MN-2007), 8.3.6.3 (MN-2022) +4 more</t>
         </is>
       </c>
     </row>
@@ -47817,11 +48017,11 @@
         </is>
       </c>
       <c r="G363" t="n">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="H363" s="8" t="inlineStr">
         <is>
-          <t>8.3.6.3 (MN-2022), 8.EE.C.7.B (CCSS-M), 8.EE.C.7.A (CCSS-M), 8.EE.7a (CCSS-M), 8.EE.7b (CCSS-M)</t>
+          <t>8.2.2.1 (MN-2007), 8.2.2.2 (MN-2007), 8.2.1.1 (MN-2007), 8.2.1.2 (MN-2007), 8.2.3.1 (MN-2007), 8.1.1.1 (MN-2007), 8.1.1.2 (MN-2007), 8.1.2.1 (MN-2007), 8.2.3.2 (MN-2007), 8.3.6.3 (MN-2022) +4 more</t>
         </is>
       </c>
     </row>
@@ -47851,11 +48051,11 @@
         </is>
       </c>
       <c r="G364" t="n">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="H364" s="8" t="inlineStr">
         <is>
-          <t>8.F.A.1 (CCSS-M), 8.3.7.2 (MN-2022), 8.3.7.6 (MN-2022), 8.F.1 (CCSS-M)</t>
+          <t>8.F.A.1 (CCSS-M), 8.2.2.1 (MN-2007), 8.2.2.2 (MN-2007), 8.2.1.1 (MN-2007), 8.2.1.2 (MN-2007), 8.2.3.1 (MN-2007), 8.1.1.1 (MN-2007), 8.1.1.2 (MN-2007), 8.1.2.1 (MN-2007), 8.2.3.2 (MN-2007) +3 more</t>
         </is>
       </c>
     </row>
@@ -47885,11 +48085,11 @@
         </is>
       </c>
       <c r="G365" t="n">
-        <v>12</v>
+        <v>26</v>
       </c>
       <c r="H365" s="8" t="inlineStr">
         <is>
-          <t>8.F.A.1 (CCSS-M), 8.F.A.2 (CCSS-M), 8.F.A.3 (CCSS-M), 8.F.B.4 (CCSS-M), 8.2.4.1 (MN-2022), 8.3.7.1 (MN-2022), 8.3.7.3 (MN-2022), 8.3.7.4 (MN-2022), 8.F.1 (CCSS-M), 8.F.2 (CCSS-M) +2 more</t>
+          <t>8.F.A.1 (CCSS-M), 8.F.A.2 (CCSS-M), 8.F.A.3 (CCSS-M), 8.F.B.4 (CCSS-M), 8.2.2.1 (MN-2007), 8.2.2.2 (MN-2007), 8.2.1.1 (MN-2007), 8.2.1.2 (MN-2007), 8.2.3.1 (MN-2007), 8.3.1.1 (MN-2007) +16 more</t>
         </is>
       </c>
     </row>
@@ -47919,11 +48119,11 @@
         </is>
       </c>
       <c r="G366" t="n">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="H366" s="8" t="inlineStr">
         <is>
-          <t>8.F.A.1 (CCSS-M), 8.F.B.4 (CCSS-M), 8.3.7.2 (MN-2022), 8.F.1 (CCSS-M), 8.F.2 (CCSS-M), 8.F.3 (CCSS-M), 8.F.4 (CCSS-M)</t>
+          <t>8.F.A.1 (CCSS-M), 8.F.B.4 (CCSS-M), 8.2.2.1 (MN-2007), 8.2.2.2 (MN-2007), 8.2.1.1 (MN-2007), 8.2.1.2 (MN-2007), 8.2.3.1 (MN-2007), 8.1.1.1 (MN-2007), 8.1.1.2 (MN-2007), 8.1.2.1 (MN-2007) +6 more</t>
         </is>
       </c>
     </row>
@@ -47987,11 +48187,11 @@
         </is>
       </c>
       <c r="G368" t="n">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="H368" s="8" t="inlineStr">
         <is>
-          <t>8.F.A.1 (CCSS-M), 8.F.B.4 (CCSS-M), 8.3.7.1 (MN-2022), 8.F.1 (CCSS-M), 8.F.2 (CCSS-M), 8.F.3 (CCSS-M), 8.F.4 (CCSS-M)</t>
+          <t>8.F.A.1 (CCSS-M), 8.F.B.4 (CCSS-M), 8.2.2.1 (MN-2007), 8.2.2.2 (MN-2007), 8.2.1.1 (MN-2007), 8.2.1.2 (MN-2007), 8.2.3.1 (MN-2007), 8.1.1.1 (MN-2007), 8.1.1.2 (MN-2007), 8.1.2.1 (MN-2007) +6 more</t>
         </is>
       </c>
     </row>
@@ -48021,11 +48221,11 @@
         </is>
       </c>
       <c r="G369" t="n">
-        <v>7</v>
+        <v>21</v>
       </c>
       <c r="H369" s="8" t="inlineStr">
         <is>
-          <t>8.F.B.5 (CCSS-M), 8.2.4.1 (MN-2022), 8.3.7.3 (MN-2022), 8.F.1 (CCSS-M), 8.F.2 (CCSS-M), 8.F.3 (CCSS-M), 8.F.4 (CCSS-M)</t>
+          <t>8.F.B.5 (CCSS-M), 8.2.2.1 (MN-2007), 8.2.2.2 (MN-2007), 8.2.1.1 (MN-2007), 8.2.1.2 (MN-2007), 8.2.3.1 (MN-2007), 8.3.1.1 (MN-2007), 8.3.1.2 (MN-2007), 8.1.1.1 (MN-2007), 8.1.1.2 (MN-2007) +11 more</t>
         </is>
       </c>
     </row>
@@ -48055,11 +48255,11 @@
         </is>
       </c>
       <c r="G370" t="n">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="H370" s="8" t="inlineStr">
         <is>
-          <t>8.F.B.4 (CCSS-M), 8.3.7.4 (MN-2022), 8.3.7.6 (MN-2022), 8.F.4 (CCSS-M)</t>
+          <t>8.F.B.4 (CCSS-M), 8.2.2.1 (MN-2007), 8.2.2.2 (MN-2007), 8.2.1.1 (MN-2007), 8.2.1.2 (MN-2007), 8.2.3.1 (MN-2007), 8.1.1.1 (MN-2007), 8.1.1.2 (MN-2007), 8.1.2.1 (MN-2007), 8.2.3.2 (MN-2007) +3 more</t>
         </is>
       </c>
     </row>
@@ -48089,11 +48289,11 @@
         </is>
       </c>
       <c r="G371" t="n">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="H371" s="8" t="inlineStr">
         <is>
-          <t>8.3.6.3 (MN-2022), 8.EE.C.7.B (CCSS-M), 8.EE.C.7.A (CCSS-M), 8.EE.7a (CCSS-M), 8.EE.7b (CCSS-M)</t>
+          <t>8.2.2.1 (MN-2007), 8.2.2.2 (MN-2007), 8.2.1.1 (MN-2007), 8.2.1.2 (MN-2007), 8.2.3.1 (MN-2007), 8.1.1.1 (MN-2007), 8.1.1.2 (MN-2007), 8.1.2.1 (MN-2007), 8.2.3.2 (MN-2007), 8.3.6.3 (MN-2022) +4 more</t>
         </is>
       </c>
     </row>
@@ -48123,11 +48323,11 @@
         </is>
       </c>
       <c r="G372" t="n">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="H372" s="8" t="inlineStr">
         <is>
-          <t>8.3.6.3 (MN-2022), 8.EE.C.7.B (CCSS-M), 8.EE.C.7.A (CCSS-M), 8.EE.7a (CCSS-M), 8.EE.7b (CCSS-M)</t>
+          <t>8.2.2.1 (MN-2007), 8.2.2.2 (MN-2007), 8.2.1.1 (MN-2007), 8.2.1.2 (MN-2007), 8.2.3.1 (MN-2007), 8.1.1.1 (MN-2007), 8.1.1.2 (MN-2007), 8.1.2.1 (MN-2007), 8.2.3.2 (MN-2007), 8.3.6.3 (MN-2022) +4 more</t>
         </is>
       </c>
     </row>
@@ -48191,11 +48391,11 @@
         </is>
       </c>
       <c r="G374" t="n">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="H374" s="8" t="inlineStr">
         <is>
-          <t>8.3.7.1 (MN-2022), 8.EE.C.7.B (CCSS-M), 8.EE.C.7.A (CCSS-M), 8.EE.7b (CCSS-M)</t>
+          <t>8.2.2.1 (MN-2007), 8.2.2.2 (MN-2007), 8.2.1.1 (MN-2007), 8.2.1.2 (MN-2007), 8.2.3.1 (MN-2007), 8.1.1.1 (MN-2007), 8.1.1.2 (MN-2007), 8.1.2.1 (MN-2007), 8.2.3.2 (MN-2007), 8.3.7.1 (MN-2022) +3 more</t>
         </is>
       </c>
     </row>
@@ -48225,11 +48425,11 @@
         </is>
       </c>
       <c r="G375" t="n">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="H375" s="8" t="inlineStr">
         <is>
-          <t>8.3.6.1 (MN-2022), 8.3.6.3 (MN-2022), 8.EE.C.7.B (CCSS-M), 8.EE.C.7.A (CCSS-M), 8.EE.7b (CCSS-M)</t>
+          <t>8.2.2.1 (MN-2007), 8.2.2.2 (MN-2007), 8.2.1.1 (MN-2007), 8.2.1.2 (MN-2007), 8.2.3.1 (MN-2007), 8.1.1.1 (MN-2007), 8.1.1.2 (MN-2007), 8.1.2.1 (MN-2007), 8.2.3.2 (MN-2007), 8.3.6.1 (MN-2022) +4 more</t>
         </is>
       </c>
     </row>
@@ -48259,11 +48459,11 @@
         </is>
       </c>
       <c r="G376" t="n">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="H376" s="8" t="inlineStr">
         <is>
-          <t>8.F.A.2 (CCSS-M), 8.F.B.4 (CCSS-M), 8.3.7.1 (MN-2022), 8.3.7.2 (MN-2022), 8.3.7.4 (MN-2022), 8.3.7.6 (MN-2022), 8.F.2 (CCSS-M), 8.F.4 (CCSS-M)</t>
+          <t>8.F.A.2 (CCSS-M), 8.F.B.4 (CCSS-M), 8.2.2.1 (MN-2007), 8.2.2.2 (MN-2007), 8.2.1.1 (MN-2007), 8.2.1.2 (MN-2007), 8.2.3.1 (MN-2007), 8.1.1.1 (MN-2007), 8.1.1.2 (MN-2007), 8.1.2.1 (MN-2007) +7 more</t>
         </is>
       </c>
     </row>
@@ -48327,11 +48527,11 @@
         </is>
       </c>
       <c r="G378" t="n">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="H378" s="8" t="inlineStr">
         <is>
-          <t>8.F.A.2 (CCSS-M), 8.F.B.4 (CCSS-M), 8.3.6.5 (MN-2022), 8.3.6.6 (MN-2022), 8.3.7.2 (MN-2022), 8.3.7.5 (MN-2022), 8.F.2 (CCSS-M), 8.F.4 (CCSS-M)</t>
+          <t>8.F.A.2 (CCSS-M), 8.F.B.4 (CCSS-M), 8.2.2.1 (MN-2007), 8.2.2.2 (MN-2007), 8.2.1.1 (MN-2007), 8.2.1.2 (MN-2007), 8.2.3.1 (MN-2007), 8.1.1.1 (MN-2007), 8.1.1.2 (MN-2007), 8.1.2.1 (MN-2007) +7 more</t>
         </is>
       </c>
     </row>
@@ -48395,11 +48595,11 @@
         </is>
       </c>
       <c r="G380" t="n">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="H380" s="8" t="inlineStr">
         <is>
-          <t>8.F.A.2 (CCSS-M), 8.F.B.4 (CCSS-M), 8.3.6.5 (MN-2022), 8.3.6.6 (MN-2022), 8.F.2 (CCSS-M), 8.F.4 (CCSS-M)</t>
+          <t>8.F.A.2 (CCSS-M), 8.F.B.4 (CCSS-M), 8.2.2.1 (MN-2007), 8.2.2.2 (MN-2007), 8.2.1.1 (MN-2007), 8.2.1.2 (MN-2007), 8.2.3.1 (MN-2007), 8.1.1.1 (MN-2007), 8.1.1.2 (MN-2007), 8.1.2.1 (MN-2007) +5 more</t>
         </is>
       </c>
     </row>
@@ -48463,11 +48663,11 @@
         </is>
       </c>
       <c r="G382" t="n">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="H382" s="8" t="inlineStr">
         <is>
-          <t>8.F.A.3 (CCSS-M), 8.F.B.5 (CCSS-M), 8.3.7.1 (MN-2022), 8.3.7.2 (MN-2022), 8.3.7.4 (MN-2022), 8.3.7.6 (MN-2022), 8.F.2 (CCSS-M), 8.F.4 (CCSS-M)</t>
+          <t>8.F.A.3 (CCSS-M), 8.F.B.5 (CCSS-M), 8.2.2.1 (MN-2007), 8.2.2.2 (MN-2007), 8.2.1.1 (MN-2007), 8.2.1.2 (MN-2007), 8.2.3.1 (MN-2007), 8.1.1.1 (MN-2007), 8.1.1.2 (MN-2007), 8.1.2.1 (MN-2007) +7 more</t>
         </is>
       </c>
     </row>
@@ -48497,11 +48697,11 @@
         </is>
       </c>
       <c r="G383" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="H383" s="8" t="inlineStr">
         <is>
-          <t>8.3.6.3 (MN-2022), 8.EE.B.8 (CCSS-M), 8.EE.8b (CCSS-M)</t>
+          <t>8.2.2.1 (MN-2007), 8.2.2.2 (MN-2007), 8.2.1.1 (MN-2007), 8.2.1.2 (MN-2007), 8.2.3.1 (MN-2007), 8.1.1.1 (MN-2007), 8.1.1.2 (MN-2007), 8.1.2.1 (MN-2007), 8.2.3.2 (MN-2007), 8.3.6.3 (MN-2022) +2 more</t>
         </is>
       </c>
     </row>
@@ -48531,11 +48731,11 @@
         </is>
       </c>
       <c r="G384" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="H384" s="8" t="inlineStr">
         <is>
-          <t>8.3.6.3 (MN-2022), 8.EE.B.7 (CCSS-M), 8.EE.7b (CCSS-M)</t>
+          <t>8.2.2.1 (MN-2007), 8.2.2.2 (MN-2007), 8.2.1.1 (MN-2007), 8.2.1.2 (MN-2007), 8.2.3.1 (MN-2007), 8.1.1.1 (MN-2007), 8.1.1.2 (MN-2007), 8.1.2.1 (MN-2007), 8.2.3.2 (MN-2007), 8.3.6.3 (MN-2022) +2 more</t>
         </is>
       </c>
     </row>
@@ -48565,11 +48765,11 @@
         </is>
       </c>
       <c r="G385" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="H385" s="8" t="inlineStr">
         <is>
-          <t>8.3.6.9 (MN-2022), 8.EE.A.8 (CCSS-M), 8.EE.8a (CCSS-M)</t>
+          <t>8.2.2.1 (MN-2007), 8.2.2.2 (MN-2007), 8.2.1.1 (MN-2007), 8.2.1.2 (MN-2007), 8.2.3.1 (MN-2007), 8.1.1.1 (MN-2007), 8.1.1.2 (MN-2007), 8.1.2.1 (MN-2007), 8.2.3.2 (MN-2007), 8.3.6.9 (MN-2022) +2 more</t>
         </is>
       </c>
     </row>
@@ -48667,11 +48867,11 @@
         </is>
       </c>
       <c r="G388" t="n">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="H388" s="8" t="inlineStr">
         <is>
-          <t>8.EE.C.8 (CCSS-M), 8.2.4.3 (MN-2022), 8.3.6.9 (MN-2022), 8.EE.B.8 (CCSS-M), 8.EE.8b (CCSS-M), 8.EE.8c (CCSS-M)</t>
+          <t>8.2.2.1 (MN-2007), 8.2.2.2 (MN-2007), 8.2.1.1 (MN-2007), 8.2.1.2 (MN-2007), 8.2.3.1 (MN-2007), 8.3.1.1 (MN-2007), 8.3.1.2 (MN-2007), 8.1.1.1 (MN-2007), 8.1.1.2 (MN-2007), 8.1.2.1 (MN-2007) +10 more</t>
         </is>
       </c>
     </row>
@@ -48837,11 +49037,11 @@
         </is>
       </c>
       <c r="G393" t="n">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="H393" s="8" t="inlineStr">
         <is>
-          <t>8.3.7.7 (MN-2022), 8.3.7.8 (MN-2022), 8.3.7.9 (MN-2022), 8.G.3 (CCSS-M)</t>
+          <t>8.2.2.1 (MN-2007), 8.2.2.2 (MN-2007), 8.2.1.1 (MN-2007), 8.2.1.2 (MN-2007), 8.2.3.1 (MN-2007), 8.1.1.1 (MN-2007), 8.1.1.2 (MN-2007), 8.1.2.1 (MN-2007), 8.2.3.2 (MN-2007), 8.3.7.7 (MN-2022) +3 more</t>
         </is>
       </c>
     </row>
@@ -48871,11 +49071,11 @@
         </is>
       </c>
       <c r="G394" t="n">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="H394" s="8" t="inlineStr">
         <is>
-          <t>8.3.7.7 (MN-2022), 8.3.7.8 (MN-2022), 8.3.7.9 (MN-2022), 8.G.3 (CCSS-M), 8.G.4 (CCSS-M)</t>
+          <t>8.2.2.1 (MN-2007), 8.2.2.2 (MN-2007), 8.2.1.1 (MN-2007), 8.2.1.2 (MN-2007), 8.2.3.1 (MN-2007), 8.1.1.1 (MN-2007), 8.1.1.2 (MN-2007), 8.1.2.1 (MN-2007), 8.2.3.2 (MN-2007), 8.3.7.7 (MN-2022) +4 more</t>
         </is>
       </c>
     </row>
@@ -49041,11 +49241,11 @@
         </is>
       </c>
       <c r="G399" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H399" s="8" t="inlineStr">
         <is>
-          <t>8.1.1.2 (MN-2022), See eBook (CCSS-M)</t>
+          <t>8.4.1.1 (MN-2007), 8.4.1.2 (MN-2007), 8.1.1.2 (MN-2022), See eBook (CCSS-M)</t>
         </is>
       </c>
     </row>
@@ -49075,11 +49275,11 @@
         </is>
       </c>
       <c r="G400" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H400" s="8" t="inlineStr">
         <is>
-          <t>8.1.1.1 (MN-2022), 8.1.1.2 (MN-2022), 8.1.1.4 (MN-2022), 8.1.1.6 (MN-2022), See eBook (CCSS-M), 8.SP.1 (CCSS-M)</t>
+          <t>8.4.1.1 (MN-2007), 8.4.1.2 (MN-2007), 8.1.1.1 (MN-2022), 8.1.1.2 (MN-2022), 8.1.1.4 (MN-2022), 8.1.1.6 (MN-2022), See eBook (CCSS-M), 8.SP.1 (CCSS-M)</t>
         </is>
       </c>
     </row>
@@ -49143,11 +49343,11 @@
         </is>
       </c>
       <c r="G402" t="n">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="H402" s="8" t="inlineStr">
         <is>
-          <t>8.2.4.1 (MN-2022), 8.2.4.2 (MN-2022), 8.3.5.8 (MN-2022), 8.3.6.5 (MN-2022), 8.3.6.6 (MN-2022), 8.3.7.1 (MN-2022), 8.3.7.3 (MN-2022), 8.3.7.6 (MN-2022), See eBook (CCSS-M), 8.F.3 (CCSS-M) +1 more</t>
+          <t>8.2.2.1 (MN-2007), 8.2.2.2 (MN-2007), 8.2.1.1 (MN-2007), 8.2.1.2 (MN-2007), 8.2.3.1 (MN-2007), 8.3.1.1 (MN-2007), 8.3.1.2 (MN-2007), 8.1.1.1 (MN-2007), 8.1.1.2 (MN-2007), 8.1.2.1 (MN-2007) +15 more</t>
         </is>
       </c>
     </row>
@@ -49279,11 +49479,11 @@
         </is>
       </c>
       <c r="G406" t="n">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="H406" s="8" t="inlineStr">
         <is>
-          <t>8.3.7.1 (MN-2022), See eBook (CCSS-M), 8.EE.5 (CCSS-M), 8.EE.6 (CCSS-M)</t>
+          <t>8.2.2.1 (MN-2007), 8.2.2.2 (MN-2007), 8.2.1.1 (MN-2007), 8.2.1.2 (MN-2007), 8.2.3.1 (MN-2007), 8.1.1.1 (MN-2007), 8.1.1.2 (MN-2007), 8.1.2.1 (MN-2007), 8.2.3.2 (MN-2007), 8.3.7.1 (MN-2022) +3 more</t>
         </is>
       </c>
     </row>
@@ -49313,11 +49513,11 @@
         </is>
       </c>
       <c r="G407" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H407" s="8" t="inlineStr">
         <is>
-          <t>8.1.1.3 (MN-2022), See eBook (CCSS-M), 8.SP.3 (CCSS-M)</t>
+          <t>8.4.1.1 (MN-2007), 8.4.1.2 (MN-2007), 8.1.1.3 (MN-2022), See eBook (CCSS-M), 8.SP.3 (CCSS-M)</t>
         </is>
       </c>
     </row>
@@ -49347,11 +49547,11 @@
         </is>
       </c>
       <c r="G408" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="H408" s="8" t="inlineStr">
         <is>
-          <t>8.1.1.1 (MN-2022), 8.1.1.3 (MN-2022), 8.1.1.4 (MN-2022), 8.1.1.5 (MN-2022), 8.1.1.6 (MN-2022), See eBook (CCSS-M), 8.SP.2 (CCSS-M), 8.SP.3 (CCSS-M)</t>
+          <t>8.4.1.1 (MN-2007), 8.4.1.2 (MN-2007), 8.1.1.1 (MN-2022), 8.1.1.3 (MN-2022), 8.1.1.4 (MN-2022), 8.1.1.5 (MN-2022), 8.1.1.6 (MN-2022), See eBook (CCSS-M), 8.SP.2 (CCSS-M), 8.SP.3 (CCSS-M)</t>
         </is>
       </c>
     </row>
@@ -49381,11 +49581,11 @@
         </is>
       </c>
       <c r="G409" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H409" s="8" t="inlineStr">
         <is>
-          <t>8.1.1.1 (MN-2022), See eBook (CCSS-M), 8.SP.4 (CCSS-M)</t>
+          <t>8.4.1.1 (MN-2007), 8.4.1.2 (MN-2007), 8.1.1.1 (MN-2022), See eBook (CCSS-M), 8.SP.4 (CCSS-M)</t>
         </is>
       </c>
     </row>
@@ -49415,11 +49615,11 @@
         </is>
       </c>
       <c r="G410" t="n">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="H410" s="8" t="inlineStr">
         <is>
-          <t>8.2.4.1 (MN-2022), 8.3.5.6 (MN-2022), 8.3.5.7 (MN-2022), 8.3.7.3 (MN-2022), See eBook (CCSS-M), 8.F.3 (CCSS-M)</t>
+          <t>8.2.2.1 (MN-2007), 8.2.2.2 (MN-2007), 8.2.1.1 (MN-2007), 8.2.1.2 (MN-2007), 8.2.3.1 (MN-2007), 8.3.1.1 (MN-2007), 8.3.1.2 (MN-2007), 8.1.1.1 (MN-2007), 8.1.1.2 (MN-2007), 8.1.2.1 (MN-2007) +10 more</t>
         </is>
       </c>
     </row>
@@ -49449,11 +49649,11 @@
         </is>
       </c>
       <c r="G411" t="n">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="H411" s="8" t="inlineStr">
         <is>
-          <t>8.3.5.6 (MN-2022), 8.3.5.7 (MN-2022), See eBook (CCSS-M), 8.EE.1 (CCSS-M)</t>
+          <t>8.2.2.1 (MN-2007), 8.2.2.2 (MN-2007), 8.2.1.1 (MN-2007), 8.2.1.2 (MN-2007), 8.2.3.1 (MN-2007), 8.1.1.1 (MN-2007), 8.1.1.2 (MN-2007), 8.1.2.1 (MN-2007), 8.2.3.2 (MN-2007), 8.3.5.6 (MN-2022) +3 more</t>
         </is>
       </c>
     </row>
@@ -49483,11 +49683,11 @@
         </is>
       </c>
       <c r="G412" t="n">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="H412" s="8" t="inlineStr">
         <is>
-          <t>8.2.4.1 (MN-2022), 8.3.5.6 (MN-2022), 8.3.5.7 (MN-2022), 8.3.7.3 (MN-2022), See eBook (CCSS-M), 8.F.3 (CCSS-M)</t>
+          <t>8.2.2.1 (MN-2007), 8.2.2.2 (MN-2007), 8.2.1.1 (MN-2007), 8.2.1.2 (MN-2007), 8.2.3.1 (MN-2007), 8.3.1.1 (MN-2007), 8.3.1.2 (MN-2007), 8.1.1.1 (MN-2007), 8.1.1.2 (MN-2007), 8.1.2.1 (MN-2007) +10 more</t>
         </is>
       </c>
     </row>
@@ -49517,11 +49717,11 @@
         </is>
       </c>
       <c r="G413" t="n">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="H413" s="8" t="inlineStr">
         <is>
-          <t>8.3.5.3 (MN-2022), 8.3.5.4 (MN-2022), 8.3.5.5 (MN-2022), See eBook (CCSS-M), 8.EE.1 (CCSS-M), 8.EE.3 (CCSS-M)</t>
+          <t>8.2.2.1 (MN-2007), 8.2.2.2 (MN-2007), 8.2.1.1 (MN-2007), 8.2.1.2 (MN-2007), 8.2.3.1 (MN-2007), 8.1.1.1 (MN-2007), 8.1.1.2 (MN-2007), 8.1.2.1 (MN-2007), 8.2.3.2 (MN-2007), 8.3.5.3 (MN-2022) +5 more</t>
         </is>
       </c>
     </row>
@@ -49585,11 +49785,11 @@
         </is>
       </c>
       <c r="G415" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="H415" s="8" t="inlineStr">
         <is>
-          <t>8.3.5.3 (MN-2022), See eBook (CCSS-M), 8.EE.1 (CCSS-M)</t>
+          <t>8.2.2.1 (MN-2007), 8.2.2.2 (MN-2007), 8.2.1.1 (MN-2007), 8.2.1.2 (MN-2007), 8.2.3.1 (MN-2007), 8.1.1.1 (MN-2007), 8.1.1.2 (MN-2007), 8.1.2.1 (MN-2007), 8.2.3.2 (MN-2007), 8.3.5.3 (MN-2022) +2 more</t>
         </is>
       </c>
     </row>
@@ -49619,11 +49819,11 @@
         </is>
       </c>
       <c r="G416" t="n">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="H416" s="8" t="inlineStr">
         <is>
-          <t>8.3.5.4 (MN-2022), 8.3.5.5 (MN-2022), See eBook (CCSS-M), 8.EE.4 (CCSS-M)</t>
+          <t>8.2.2.1 (MN-2007), 8.2.2.2 (MN-2007), 8.2.1.1 (MN-2007), 8.2.1.2 (MN-2007), 8.2.3.1 (MN-2007), 8.1.1.1 (MN-2007), 8.1.1.2 (MN-2007), 8.1.2.1 (MN-2007), 8.2.3.2 (MN-2007), 8.3.5.4 (MN-2022) +3 more</t>
         </is>
       </c>
     </row>
@@ -49653,11 +49853,11 @@
         </is>
       </c>
       <c r="G417" t="n">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="H417" s="8" t="inlineStr">
         <is>
-          <t>8.3.7.3 (MN-2022), 8.3.7.6 (MN-2022), See eBook (CCSS-M), 8.F.1 (CCSS-M), 8.F.3 (CCSS-M), 8.F.5 (CCSS-M)</t>
+          <t>8.2.2.1 (MN-2007), 8.2.2.2 (MN-2007), 8.2.1.1 (MN-2007), 8.2.1.2 (MN-2007), 8.2.3.1 (MN-2007), 8.1.1.1 (MN-2007), 8.1.1.2 (MN-2007), 8.1.2.1 (MN-2007), 8.2.3.2 (MN-2007), 8.3.7.3 (MN-2022) +5 more</t>
         </is>
       </c>
     </row>
@@ -49687,11 +49887,11 @@
         </is>
       </c>
       <c r="G418" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="H418" s="8" t="inlineStr">
         <is>
-          <t>8.2.3.1 (MN-2022), 8.2.3.2 (MN-2022), 8.2.3.3 (MN-2022), See eBook (CCSS-M), 8.G.5 (CCSS-M)</t>
+          <t>8.3.1.1 (MN-2007), 8.3.1.2 (MN-2007), 8.3.2.1 (MN-2007), 8.3.2.2 (MN-2007), 8.3.3.1 (MN-2007), 8.2.3.1 (MN-2022), 8.2.3.2 (MN-2022), 8.2.3.3 (MN-2022), See eBook (CCSS-M), 8.G.5 (CCSS-M)</t>
         </is>
       </c>
     </row>
@@ -49721,11 +49921,11 @@
         </is>
       </c>
       <c r="G419" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="H419" s="8" t="inlineStr">
         <is>
-          <t>8.2.3.1 (MN-2022), 8.2.3.2 (MN-2022), See eBook (CCSS-M), 8.G.5 (CCSS-M)</t>
+          <t>8.3.1.1 (MN-2007), 8.3.1.2 (MN-2007), 8.3.2.1 (MN-2007), 8.3.2.2 (MN-2007), 8.3.3.1 (MN-2007), 8.2.3.1 (MN-2022), 8.2.3.2 (MN-2022), See eBook (CCSS-M), 8.G.5 (CCSS-M)</t>
         </is>
       </c>
     </row>
@@ -49755,11 +49955,11 @@
         </is>
       </c>
       <c r="G420" t="n">
-        <v>5</v>
+        <v>19</v>
       </c>
       <c r="H420" s="8" t="inlineStr">
         <is>
-          <t>8.2.3.1 (MN-2022), 8.3.5.2 (MN-2022), 8.3.6.4 (MN-2022), See eBook (CCSS-M), 8.G.5 (CCSS-M)</t>
+          <t>8.2.2.1 (MN-2007), 8.2.2.2 (MN-2007), 8.2.1.1 (MN-2007), 8.2.1.2 (MN-2007), 8.2.3.1 (MN-2007), 8.3.1.1 (MN-2007), 8.3.1.2 (MN-2007), 8.1.1.1 (MN-2007), 8.1.1.2 (MN-2007), 8.1.2.1 (MN-2007) +9 more</t>
         </is>
       </c>
     </row>
@@ -49789,11 +49989,11 @@
         </is>
       </c>
       <c r="G421" t="n">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="H421" s="8" t="inlineStr">
         <is>
-          <t>8.3.5.1 (MN-2022), 8.3.5.2 (MN-2022), 8.3.6.4 (MN-2022), See eBook (CCSS-M), 8.G.5 (CCSS-M)</t>
+          <t>8.2.2.1 (MN-2007), 8.2.2.2 (MN-2007), 8.2.1.1 (MN-2007), 8.2.1.2 (MN-2007), 8.2.3.1 (MN-2007), 8.1.1.1 (MN-2007), 8.1.1.2 (MN-2007), 8.1.2.1 (MN-2007), 8.2.3.2 (MN-2007), 8.3.5.1 (MN-2022) +4 more</t>
         </is>
       </c>
     </row>
@@ -50061,11 +50261,11 @@
         </is>
       </c>
       <c r="G429" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="H429" s="8" t="inlineStr">
         <is>
-          <t>8.3.6.7 (MN-2022), See eBook (CCSS-M), 8.EE.2 (CCSS-M)</t>
+          <t>8.2.2.1 (MN-2007), 8.2.2.2 (MN-2007), 8.2.1.1 (MN-2007), 8.2.1.2 (MN-2007), 8.2.3.1 (MN-2007), 8.1.1.1 (MN-2007), 8.1.1.2 (MN-2007), 8.1.2.1 (MN-2007), 8.2.3.2 (MN-2007), 8.3.6.7 (MN-2022) +2 more</t>
         </is>
       </c>
     </row>
@@ -50095,11 +50295,11 @@
         </is>
       </c>
       <c r="G430" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="H430" s="8" t="inlineStr">
         <is>
-          <t>8.3.6.7 (MN-2022), See eBook (CCSS-M), 8.G.9 (CCSS-M)</t>
+          <t>8.2.2.1 (MN-2007), 8.2.2.2 (MN-2007), 8.2.1.1 (MN-2007), 8.2.1.2 (MN-2007), 8.2.3.1 (MN-2007), 8.1.1.1 (MN-2007), 8.1.1.2 (MN-2007), 8.1.2.1 (MN-2007), 8.2.3.2 (MN-2007), 8.3.6.7 (MN-2022) +2 more</t>
         </is>
       </c>
     </row>
@@ -50131,11 +50331,11 @@
         </is>
       </c>
       <c r="G431" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="H431" s="8" t="inlineStr">
         <is>
-          <t>8.3.6.8 (MN-2022), See eBook (CCSS-M), 8.G.9 (CCSS-M)</t>
+          <t>8.2.2.1 (MN-2007), 8.2.2.2 (MN-2007), 8.2.1.1 (MN-2007), 8.2.1.2 (MN-2007), 8.2.3.1 (MN-2007), 8.1.1.1 (MN-2007), 8.1.1.2 (MN-2007), 8.1.2.1 (MN-2007), 8.2.3.2 (MN-2007), 8.3.6.8 (MN-2022) +2 more</t>
         </is>
       </c>
     </row>
@@ -50233,11 +50433,11 @@
         </is>
       </c>
       <c r="G434" t="n">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="H434" s="8" t="inlineStr">
         <is>
-          <t>8.3.6.9 (MN-2022), See eBook (CCSS-M)</t>
+          <t>8.2.2.1 (MN-2007), 8.2.2.2 (MN-2007), 8.2.1.1 (MN-2007), 8.2.1.2 (MN-2007), 8.2.3.1 (MN-2007), 8.1.1.1 (MN-2007), 8.1.1.2 (MN-2007), 8.1.2.1 (MN-2007), 8.2.3.2 (MN-2007), 8.3.6.9 (MN-2022) +1 more</t>
         </is>
       </c>
     </row>
@@ -50331,11 +50531,11 @@
       </c>
       <c r="F437" s="8" t="inlineStr"/>
       <c r="G437" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="H437" s="8" t="inlineStr">
         <is>
-          <t>8.3.6.9 (MN-2022)</t>
+          <t>8.2.2.1 (MN-2007), 8.2.2.2 (MN-2007), 8.2.1.1 (MN-2007), 8.2.1.2 (MN-2007), 8.2.3.1 (MN-2007), 8.1.1.1 (MN-2007), 8.1.1.2 (MN-2007), 8.1.2.1 (MN-2007), 8.2.3.2 (MN-2007), 8.3.6.9 (MN-2022)</t>
         </is>
       </c>
     </row>
@@ -50361,11 +50561,11 @@
         </is>
       </c>
       <c r="G438" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="H438" s="8" t="inlineStr">
         <is>
-          <t>9.3.6.7 (MN-2022), 9.3.7.1 (MN-2022), 9.3.7.2 (MN-2022), 9.3.7.7 (MN-2022)</t>
+          <t>9.3.6.7 (MN-2022), 9.3.7.1 (MN-2022), 9.3.7.2 (MN-2022), 9.3.7.7 (MN-2022), 8.EE.C.7.A (CCSS-M), 7.EE.A.1.A (CCSS-M), 8.EE.A.8 (CCSS-M)</t>
         </is>
       </c>
     </row>
@@ -50391,11 +50591,11 @@
         </is>
       </c>
       <c r="G439" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="H439" s="8" t="inlineStr">
         <is>
-          <t>9.3.7.1 (MN-2022), 9.3.7.2 (MN-2022), 9.3.7.7 (MN-2022)</t>
+          <t>9.3.7.1 (MN-2022), 9.3.7.2 (MN-2022), 9.3.7.7 (MN-2022), 8.EE.C.7.A (CCSS-M), 7.EE.A.1.A (CCSS-M), 8.EE.A.8 (CCSS-M)</t>
         </is>
       </c>
     </row>
@@ -50421,11 +50621,11 @@
         </is>
       </c>
       <c r="G440" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="H440" s="8" t="inlineStr">
         <is>
-          <t>9.2.3.6 (MN-2022), 9.3.7.1 (MN-2022), 9.3.7.7 (MN-2022)</t>
+          <t>9.2.3.6 (MN-2022), 9.3.7.1 (MN-2022), 9.3.7.7 (MN-2022), 5.NF.A.1 (CCSS-M), 8.EE.C.7.A (CCSS-M), 8.EE.A.8 (CCSS-M)</t>
         </is>
       </c>
     </row>
@@ -50477,11 +50677,11 @@
         </is>
       </c>
       <c r="G442" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="H442" s="8" t="inlineStr">
         <is>
-          <t>9.3.5.8 (MN-2022), 9.3.6.1 (MN-2022), 9.3.7.1 (MN-2022)</t>
+          <t>9.3.5.8 (MN-2022), 9.3.6.1 (MN-2022), 9.3.7.1 (MN-2022), 7.SP.8a (CCSS-M), 7.EE.3 (CCSS-M), 8.EE.C.7.A (CCSS-M)</t>
         </is>
       </c>
     </row>
@@ -50507,11 +50707,11 @@
         </is>
       </c>
       <c r="G443" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H443" s="8" t="inlineStr">
         <is>
-          <t>9.3.7.1 (MN-2022)</t>
+          <t>9.3.7.1 (MN-2022), 8.EE.C.7.A (CCSS-M)</t>
         </is>
       </c>
     </row>
@@ -50537,11 +50737,11 @@
         </is>
       </c>
       <c r="G444" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H444" s="8" t="inlineStr">
         <is>
-          <t>9.3.7.1 (MN-2022)</t>
+          <t>9.3.7.1 (MN-2022), 8.EE.C.7.A (CCSS-M)</t>
         </is>
       </c>
     </row>
@@ -50567,11 +50767,11 @@
         </is>
       </c>
       <c r="G445" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="H445" s="8" t="inlineStr">
         <is>
-          <t>9.3.7.1 (MN-2022), 9.3.7.4 (MN-2022), 9.3.7.5 (MN-2022)</t>
+          <t>9.3.7.1 (MN-2022), 9.3.7.4 (MN-2022), 9.3.7.5 (MN-2022), 8.EE.C.7.A (CCSS-M), 7.EE.B.4.B (CCSS-M), 8.EE.B.8 (CCSS-M)</t>
         </is>
       </c>
     </row>
@@ -50597,11 +50797,11 @@
         </is>
       </c>
       <c r="G446" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H446" s="8" t="inlineStr">
         <is>
-          <t>9.3.7.4 (MN-2022), 9.3.7.5 (MN-2022)</t>
+          <t>9.3.7.4 (MN-2022), 9.3.7.5 (MN-2022), 7.EE.B.4.B (CCSS-M), 8.EE.B.8 (CCSS-M)</t>
         </is>
       </c>
     </row>
@@ -50627,11 +50827,11 @@
         </is>
       </c>
       <c r="G447" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="H447" s="8" t="inlineStr">
         <is>
-          <t>9.3.5.5 (MN-2022), 9.3.7.1 (MN-2022), 9.3.7.4 (MN-2022), 9.3.7.5 (MN-2022), 9.3.7.7 (MN-2022)</t>
+          <t>9.3.5.5 (MN-2022), 9.3.7.1 (MN-2022), 9.3.7.4 (MN-2022), 9.3.7.5 (MN-2022), 9.3.7.7 (MN-2022), 8.EE.C.7.A (CCSS-M), 7.EE.B.4.B (CCSS-M), 8.EE.B.8 (CCSS-M), 8.EE.A.8 (CCSS-M)</t>
         </is>
       </c>
     </row>
@@ -50657,11 +50857,11 @@
         </is>
       </c>
       <c r="G448" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="H448" s="8" t="inlineStr">
         <is>
-          <t>9.1.1.6 (MN-2022), 9.1.1.11 (MN-2022), 9.2.3.6 (MN-2022), 9.3.5.6 (MN-2022), 9.3.7.1 (MN-2022)</t>
+          <t>9.1.1.6 (MN-2022), 9.1.1.11 (MN-2022), 9.2.3.6 (MN-2022), 9.3.5.6 (MN-2022), 9.3.7.1 (MN-2022), 6.RP.A.3.C (CCSS-M), 5.NF.A.1 (CCSS-M), 7.Sp.8a (CCSS-M), 8.EE.C.7.A (CCSS-M)</t>
         </is>
       </c>
     </row>
@@ -50687,11 +50887,11 @@
         </is>
       </c>
       <c r="G449" t="n">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="H449" s="8" t="inlineStr">
         <is>
-          <t>9.1.1.5 (MN-2022), 9.1.1.6 (MN-2022), 9.1.1.8 (MN-2022), 9.1.1.11 (MN-2022), 9.1.1.15 (MN-2022), 9.2.3.6 (MN-2022), 9.3.5.6 (MN-2022)</t>
+          <t>9.1.1.5 (MN-2022), 9.1.1.6 (MN-2022), 9.1.1.8 (MN-2022), 9.1.1.11 (MN-2022), 9.1.1.15 (MN-2022), 9.2.3.6 (MN-2022), 9.3.5.6 (MN-2022), 6.EE.A.3 (CCSS-M), 6.RP.A.3.C (CCSS-M), 6.NS.C.6.B (CCSS-M) +3 more</t>
         </is>
       </c>
     </row>
@@ -50717,11 +50917,11 @@
         </is>
       </c>
       <c r="G450" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="H450" s="8" t="inlineStr">
         <is>
-          <t>9.3.7.2 (MN-2022), 9.3.7.3 (MN-2022), 9.3.7.6 (MN-2022), 9.3.7.7 (MN-2022), 9.3.7.10 (MN-2022)</t>
+          <t>9.3.7.2 (MN-2022), 9.3.7.3 (MN-2022), 9.3.7.6 (MN-2022), 9.3.7.7 (MN-2022), 9.3.7.10 (MN-2022), 7.EE.A.1.A (CCSS-M), 7.EE.A.1.B (CCSS-M), 8.EE.B.7 (CCSS-M), 8.EE.A.8 (CCSS-M), 8.G.2 (CCSS-M)</t>
         </is>
       </c>
     </row>
@@ -50747,11 +50947,11 @@
         </is>
       </c>
       <c r="G451" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="H451" s="8" t="inlineStr">
         <is>
-          <t>9.2.3.6 (MN-2022), 9.3.5.6 (MN-2022), 9.3.7.1 (MN-2022)</t>
+          <t>9.2.3.6 (MN-2022), 9.3.5.6 (MN-2022), 9.3.7.1 (MN-2022), 5.NF.A.1 (CCSS-M), 7.Sp.8a (CCSS-M), 8.EE.C.7.A (CCSS-M)</t>
         </is>
       </c>
     </row>
@@ -50777,11 +50977,11 @@
         </is>
       </c>
       <c r="G452" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="H452" s="8" t="inlineStr">
         <is>
-          <t>9.2.3.6 (MN-2022), 9.3.7.1 (MN-2022), 9.3.7.2 (MN-2022), 9.3.7.6 (MN-2022), 9.3.7.7 (MN-2022), 9.3.7.8 (MN-2022)</t>
+          <t>9.2.3.6 (MN-2022), 9.3.7.1 (MN-2022), 9.3.7.2 (MN-2022), 9.3.7.6 (MN-2022), 9.3.7.7 (MN-2022), 9.3.7.8 (MN-2022), 5.NF.A.1 (CCSS-M), 8.EE.C.7.A (CCSS-M), 7.EE.A.1.A (CCSS-M), 8.EE.B.7 (CCSS-M) +2 more</t>
         </is>
       </c>
     </row>
@@ -50807,11 +51007,11 @@
         </is>
       </c>
       <c r="G453" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="H453" s="8" t="inlineStr">
         <is>
-          <t>9.3.5.2 (MN-2022), 9.3.5.6 (MN-2022), 9.3.6.8 (MN-2022), 9.3.7.1 (MN-2022), 9.3.7.2 (MN-2022)</t>
+          <t>9.3.5.2 (MN-2022), 9.3.5.6 (MN-2022), 9.3.6.8 (MN-2022), 9.3.7.1 (MN-2022), 9.3.7.2 (MN-2022), 7.Sp.8a (CCSS-M), MP8 (CCSS-M), 8.EE.C.7.A (CCSS-M), 7.EE.A.1.A (CCSS-M)</t>
         </is>
       </c>
     </row>
@@ -50837,11 +51037,11 @@
         </is>
       </c>
       <c r="G454" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H454" s="8" t="inlineStr">
         <is>
-          <t>9.2.3.6 (MN-2022), 9.3.7.1 (MN-2022)</t>
+          <t>9.2.3.6 (MN-2022), 9.3.7.1 (MN-2022), 5.NF.A.1 (CCSS-M), 8.EE.C.7.A (CCSS-M)</t>
         </is>
       </c>
     </row>
@@ -50867,11 +51067,11 @@
         </is>
       </c>
       <c r="G455" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H455" s="8" t="inlineStr">
         <is>
-          <t>9.3.5.7 (MN-2022), 9.3.5.8 (MN-2022), 9.3.6.2 (MN-2022), 9.3.6.4 (MN-2022)</t>
+          <t>9.3.5.7 (MN-2022), 9.3.5.8 (MN-2022), 9.3.6.2 (MN-2022), 9.3.6.4 (MN-2022), 7.SP.8a (CCSS-M), 7.EE.4b (CCSS-M)</t>
         </is>
       </c>
     </row>
@@ -50897,11 +51097,11 @@
         </is>
       </c>
       <c r="G456" t="n">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="H456" s="8" t="inlineStr">
         <is>
-          <t>9.2.3.6 (MN-2022), 9.3.5.7 (MN-2022), 9.3.5.8 (MN-2022), 9.3.6.2 (MN-2022), 9.3.6.3 (MN-2022), 9.3.6.5 (MN-2022), 9.3.7.1 (MN-2022), 9.3.7.2 (MN-2022), 9.3.7.7 (MN-2022)</t>
+          <t>9.2.3.6 (MN-2022), 9.3.5.7 (MN-2022), 9.3.5.8 (MN-2022), 9.3.6.2 (MN-2022), 9.3.6.3 (MN-2022), 9.3.6.5 (MN-2022), 9.3.7.1 (MN-2022), 9.3.7.2 (MN-2022), 9.3.7.7 (MN-2022), 5.NF.A.1 (CCSS-M) +6 more</t>
         </is>
       </c>
     </row>
@@ -50927,11 +51127,11 @@
         </is>
       </c>
       <c r="G457" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H457" s="8" t="inlineStr">
         <is>
-          <t>9.3.6.3 (MN-2022), 9.3.6.5 (MN-2022)</t>
+          <t>9.3.6.3 (MN-2022), 9.3.6.5 (MN-2022), 7.EE.4a (CCSS-M), see ebook (CCSS-M)</t>
         </is>
       </c>
     </row>
@@ -50957,11 +51157,11 @@
         </is>
       </c>
       <c r="G458" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H458" s="8" t="inlineStr">
         <is>
-          <t>9.3.7.1 (MN-2022)</t>
+          <t>9.3.7.1 (MN-2022), 8.EE.C.7.A (CCSS-M)</t>
         </is>
       </c>
     </row>
@@ -51013,11 +51213,11 @@
         </is>
       </c>
       <c r="G460" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H460" s="8" t="inlineStr">
         <is>
-          <t>9.3.7.1 (MN-2022)</t>
+          <t>9.3.7.1 (MN-2022), 8.EE.C.7.A (CCSS-M)</t>
         </is>
       </c>
     </row>
@@ -51043,11 +51243,11 @@
         </is>
       </c>
       <c r="G461" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H461" s="8" t="inlineStr">
         <is>
-          <t>9.1.2.5 (MN-2022)</t>
+          <t>9.1.2.5 (MN-2022), 6.NS.3 (CCSS-M)</t>
         </is>
       </c>
     </row>
@@ -51073,11 +51273,11 @@
         </is>
       </c>
       <c r="G462" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H462" s="8" t="inlineStr">
         <is>
-          <t>9.3.5.3 (MN-2022), 9.3.5.7 (MN-2022), 9.3.5.8 (MN-2022)</t>
+          <t>9.3.5.3 (MN-2022), 9.3.5.7 (MN-2022), 9.3.5.8 (MN-2022), 7.SP.8b (CCSS-M), 7.SP.8a (CCSS-M)</t>
         </is>
       </c>
     </row>
@@ -51129,11 +51329,11 @@
         </is>
       </c>
       <c r="G464" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H464" s="8" t="inlineStr">
         <is>
-          <t>9.3.5.7 (MN-2022), 9.3.5.8 (MN-2022)</t>
+          <t>9.3.5.7 (MN-2022), 9.3.5.8 (MN-2022), 7.SP.8a (CCSS-M)</t>
         </is>
       </c>
     </row>
@@ -51159,11 +51359,11 @@
         </is>
       </c>
       <c r="G465" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="H465" s="8" t="inlineStr">
         <is>
-          <t>9.3.7.2 (MN-2022), 9.3.7.3 (MN-2022), 9.3.7.9 (MN-2022)</t>
+          <t>9.3.7.2 (MN-2022), 9.3.7.3 (MN-2022), 9.3.7.9 (MN-2022), 7.EE.A.1.A (CCSS-M), 7.EE.A.1.B (CCSS-M), 8.G.C.1 (CCSS-M)</t>
         </is>
       </c>
     </row>
@@ -51189,11 +51389,11 @@
         </is>
       </c>
       <c r="G466" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="H466" s="8" t="inlineStr">
         <is>
-          <t>9.1.1.7 (MN-2022), 9.1.1.9 (MN-2022), 9.1.1.10 (MN-2022), 9.1.1.13 (MN-2022)</t>
+          <t>9.1.1.7 (MN-2022), 9.1.1.9 (MN-2022), 9.1.1.10 (MN-2022), 9.1.1.13 (MN-2022), 6.NS.C.6.A (CCSS-M), 6.NS.C.7.A (CCSS-M), 6.NS.C.7.B (CCSS-M), 6.NS.C.7.D (CCSS-M)</t>
         </is>
       </c>
     </row>
@@ -51219,11 +51419,11 @@
         </is>
       </c>
       <c r="G467" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H467" s="8" t="inlineStr">
         <is>
-          <t>9.2.3.7 (MN-2022), 9.3.7.1 (MN-2022)</t>
+          <t>9.2.3.7 (MN-2022), 9.3.7.1 (MN-2022), 8.EE.C.7.A (CCSS-M)</t>
         </is>
       </c>
     </row>
@@ -51249,11 +51449,11 @@
         </is>
       </c>
       <c r="G468" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="H468" s="8" t="inlineStr">
         <is>
-          <t>9.3.6.5 (MN-2022), 9.3.7.2 (MN-2022), 9.3.7.6 (MN-2022), 9.3.7.7 (MN-2022), 9.3.7.10 (MN-2022)</t>
+          <t>9.3.6.5 (MN-2022), 9.3.7.2 (MN-2022), 9.3.7.6 (MN-2022), 9.3.7.7 (MN-2022), 9.3.7.10 (MN-2022), see ebook (CCSS-M), 7.EE.A.1.A (CCSS-M), 8.EE.B.7 (CCSS-M), 8.EE.A.8 (CCSS-M), 8.G.2 (CCSS-M)</t>
         </is>
       </c>
     </row>
@@ -51279,11 +51479,11 @@
         </is>
       </c>
       <c r="G469" t="n">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="H469" s="8" t="inlineStr">
         <is>
-          <t>9.3.5.6 (MN-2022), 9.3.5.7 (MN-2022), 9.3.5.8 (MN-2022), 9.3.6.2 (MN-2022), 9.3.6.3 (MN-2022), 9.3.6.5 (MN-2022), 9.3.7.1 (MN-2022), 9.3.7.2 (MN-2022), 9.3.7.3 (MN-2022)</t>
+          <t>9.3.5.6 (MN-2022), 9.3.5.7 (MN-2022), 9.3.5.8 (MN-2022), 9.3.6.2 (MN-2022), 9.3.6.3 (MN-2022), 9.3.6.5 (MN-2022), 9.3.7.1 (MN-2022), 9.3.7.2 (MN-2022), 9.3.7.3 (MN-2022), 7.Sp.8a (CCSS-M) +6 more</t>
         </is>
       </c>
     </row>
@@ -51309,11 +51509,11 @@
         </is>
       </c>
       <c r="G470" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="H470" s="8" t="inlineStr">
         <is>
-          <t>9.3.5.7 (MN-2022), 9.3.5.8 (MN-2022), 9.3.6.1 (MN-2022), 9.3.6.4 (MN-2022), 9.3.7.1 (MN-2022)</t>
+          <t>9.3.5.7 (MN-2022), 9.3.5.8 (MN-2022), 9.3.6.1 (MN-2022), 9.3.6.4 (MN-2022), 9.3.7.1 (MN-2022), 7.SP.8a (CCSS-M), 7.EE.3 (CCSS-M), 7.EE.4b (CCSS-M), 8.EE.C.7.A (CCSS-M)</t>
         </is>
       </c>
     </row>
@@ -51339,11 +51539,11 @@
         </is>
       </c>
       <c r="G471" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H471" s="8" t="inlineStr">
         <is>
-          <t>9.3.7.1 (MN-2022)</t>
+          <t>9.3.7.1 (MN-2022), 8.EE.C.7.A (CCSS-M)</t>
         </is>
       </c>
     </row>
@@ -51369,11 +51569,11 @@
         </is>
       </c>
       <c r="G472" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H472" s="8" t="inlineStr">
         <is>
-          <t>9.3.5.9 (MN-2022), 9.3.7.9 (MN-2022)</t>
+          <t>9.3.5.9 (MN-2022), 9.3.7.9 (MN-2022), 8.G.C.1 (CCSS-M)</t>
         </is>
       </c>
     </row>
@@ -51399,11 +51599,11 @@
         </is>
       </c>
       <c r="G473" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H473" s="8" t="inlineStr">
         <is>
-          <t>9.3.6.5 (MN-2022)</t>
+          <t>9.3.6.5 (MN-2022), see ebook (CCSS-M)</t>
         </is>
       </c>
     </row>
@@ -51481,11 +51681,11 @@
         </is>
       </c>
       <c r="G476" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="H476" s="8" t="inlineStr">
         <is>
-          <t>9.3.7.1 (MN-2022), 9.3.7.2 (MN-2022), 9.3.7.3 (MN-2022)</t>
+          <t>9.3.7.1 (MN-2022), 9.3.7.2 (MN-2022), 9.3.7.3 (MN-2022), 8.EE.C.7.A (CCSS-M), 7.EE.A.1.A (CCSS-M), 7.EE.A.1.B (CCSS-M)</t>
         </is>
       </c>
     </row>
@@ -51511,11 +51711,11 @@
         </is>
       </c>
       <c r="G477" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H477" s="8" t="inlineStr">
         <is>
-          <t>9.2.3.7 (MN-2022), 9.3.5.6 (MN-2022), 9.3.7.1 (MN-2022)</t>
+          <t>9.2.3.7 (MN-2022), 9.3.5.6 (MN-2022), 9.3.7.1 (MN-2022), 7.Sp.8a (CCSS-M), 8.EE.C.7.A (CCSS-M)</t>
         </is>
       </c>
     </row>
@@ -51541,11 +51741,11 @@
         </is>
       </c>
       <c r="G478" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H478" s="8" t="inlineStr">
         <is>
-          <t>9.3.7.3 (MN-2022), 9.3.7.9 (MN-2022)</t>
+          <t>9.3.7.3 (MN-2022), 9.3.7.9 (MN-2022), 7.EE.A.1.B (CCSS-M), 8.G.C.1 (CCSS-M)</t>
         </is>
       </c>
     </row>
@@ -51571,11 +51771,11 @@
         </is>
       </c>
       <c r="G479" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H479" s="8" t="inlineStr">
         <is>
-          <t>9.3.7.2 (MN-2022), 9.3.7.7 (MN-2022)</t>
+          <t>9.3.7.2 (MN-2022), 9.3.7.7 (MN-2022), 7.EE.A.1.A (CCSS-M), 8.EE.A.8 (CCSS-M)</t>
         </is>
       </c>
     </row>
@@ -51601,11 +51801,11 @@
         </is>
       </c>
       <c r="G480" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H480" s="8" t="inlineStr">
         <is>
-          <t>9.3.5.3 (MN-2022), 9.3.6.5 (MN-2022)</t>
+          <t>9.3.5.3 (MN-2022), 9.3.6.5 (MN-2022), 7.SP.8b (CCSS-M), see ebook (CCSS-M)</t>
         </is>
       </c>
     </row>
@@ -51653,11 +51853,11 @@
         </is>
       </c>
       <c r="G482" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="H482" s="8" t="inlineStr">
         <is>
-          <t>9.1.1.1 (MN-2022), 9.1.1.2 (MN-2022), 9.1.1.3 (MN-2022), 9.1.1.4 (MN-2022), 9.1.1.5 (MN-2022), 9.1.1.12 (MN-2022), 9.1.1.14 (MN-2022), 9.1.1.15 (MN-2022)</t>
+          <t>9.1.1.1 (MN-2022), 9.1.1.2 (MN-2022), 9.1.1.3 (MN-2022), 9.1.1.4 (MN-2022), 9.1.1.5 (MN-2022), 9.1.1.12 (MN-2022), 9.1.1.14 (MN-2022), 9.1.1.15 (MN-2022), MP 7 (CCSS-M), MP 1 (CCSS-M) +6 more</t>
         </is>
       </c>
     </row>
@@ -51683,11 +51883,11 @@
         </is>
       </c>
       <c r="G483" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H483" s="8" t="inlineStr">
         <is>
-          <t>9.1.1.5 (MN-2022)</t>
+          <t>9.1.1.5 (MN-2022), 6.EE.A.3 (CCSS-M)</t>
         </is>
       </c>
     </row>
@@ -51709,11 +51909,11 @@
       <c r="E484" s="7" t="n"/>
       <c r="F484" s="8" t="inlineStr"/>
       <c r="G484" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="H484" s="8" t="inlineStr">
         <is>
-          <t>9.1.1.7 (MN-2022), 9.1.1.9 (MN-2022), 9.1.1.10 (MN-2022), 9.1.1.13 (MN-2022)</t>
+          <t>9.1.1.7 (MN-2022), 9.1.1.9 (MN-2022), 9.1.1.10 (MN-2022), 9.1.1.13 (MN-2022), 6.NS.C.6.A (CCSS-M), 6.NS.C.7.A (CCSS-M), 6.NS.C.7.B (CCSS-M), 6.NS.C.7.D (CCSS-M)</t>
         </is>
       </c>
     </row>
@@ -51761,11 +51961,11 @@
         </is>
       </c>
       <c r="G486" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="H486" s="8" t="inlineStr">
         <is>
-          <t>9.3.7.4 (MN-2022), 9.3.7.5 (MN-2022), 9.3.7.8 (MN-2022)</t>
+          <t>9.3.7.4 (MN-2022), 9.3.7.5 (MN-2022), 9.3.7.8 (MN-2022), 7.EE.B.4.B (CCSS-M), 8.EE.B.8 (CCSS-M), 8.G.B.1 (CCSS-M)</t>
         </is>
       </c>
     </row>
@@ -51787,11 +51987,11 @@
       <c r="E487" s="7" t="n"/>
       <c r="F487" s="8" t="inlineStr"/>
       <c r="G487" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H487" s="8" t="inlineStr">
         <is>
-          <t>9.1.2.6 (MN-2022), 9.3.7.8 (MN-2022)</t>
+          <t>9.1.2.6 (MN-2022), 9.3.7.8 (MN-2022), 8.G.B.1 (CCSS-M)</t>
         </is>
       </c>
     </row>
@@ -51817,11 +52017,11 @@
         </is>
       </c>
       <c r="G488" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H488" s="8" t="inlineStr">
         <is>
-          <t>9.3.5.7 (MN-2022), 9.3.5.8 (MN-2022)</t>
+          <t>9.3.5.7 (MN-2022), 9.3.5.8 (MN-2022), 7.SP.8a (CCSS-M)</t>
         </is>
       </c>
     </row>
@@ -51847,11 +52047,11 @@
         </is>
       </c>
       <c r="G489" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H489" s="8" t="inlineStr">
         <is>
-          <t>9.3.7.1 (MN-2022)</t>
+          <t>9.3.7.1 (MN-2022), 8.EE.C.7.A (CCSS-M)</t>
         </is>
       </c>
     </row>
@@ -51877,11 +52077,11 @@
         </is>
       </c>
       <c r="G490" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H490" s="8" t="inlineStr">
         <is>
-          <t>9.1.2.4 (MN-2022)</t>
+          <t>9.1.2.4 (MN-2022), 6.RP.3c (CCSS-M)</t>
         </is>
       </c>
     </row>
@@ -51907,11 +52107,11 @@
         </is>
       </c>
       <c r="G491" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H491" s="8" t="inlineStr">
         <is>
-          <t>9.1.1.8 (MN-2022)</t>
+          <t>9.1.1.8 (MN-2022), 6.NS.C.6.B (CCSS-M)</t>
         </is>
       </c>
     </row>
@@ -51959,11 +52159,11 @@
         </is>
       </c>
       <c r="G493" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H493" s="8" t="inlineStr">
         <is>
-          <t>9.3.7.9 (MN-2022)</t>
+          <t>9.3.7.9 (MN-2022), 8.G.C.1 (CCSS-M)</t>
         </is>
       </c>
     </row>
@@ -52015,11 +52215,11 @@
         </is>
       </c>
       <c r="G495" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="H495" s="8" t="inlineStr">
         <is>
-          <t>9.3.6.3 (MN-2022), 9.3.7.2 (MN-2022), 9.3.7.3 (MN-2022), 9.3.7.6 (MN-2022), 9.3.7.10 (MN-2022)</t>
+          <t>9.3.6.3 (MN-2022), 9.3.7.2 (MN-2022), 9.3.7.3 (MN-2022), 9.3.7.6 (MN-2022), 9.3.7.10 (MN-2022), 7.EE.4a (CCSS-M), 7.EE.A.1.A (CCSS-M), 7.EE.A.1.B (CCSS-M), 8.EE.B.7 (CCSS-M), 8.G.2 (CCSS-M)</t>
         </is>
       </c>
     </row>
@@ -52067,11 +52267,11 @@
         </is>
       </c>
       <c r="G497" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H497" s="8" t="inlineStr">
         <is>
-          <t>9.2.4.6 (MN-2022), 9.2.4.12 (MN-2022)</t>
+          <t>9.2.4.6 (MN-2022), 9.2.4.12 (MN-2022), 7.RP.A.2.D (CCSS-M), 7.SP.7a (CCSS-M)</t>
         </is>
       </c>
     </row>
@@ -52097,11 +52297,11 @@
         </is>
       </c>
       <c r="G498" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="H498" s="8" t="inlineStr">
         <is>
-          <t>9.2.4.1 (MN-2022), 9.2.4.12 (MN-2022), 9.2.4.13 (MN-2022), 9.2.4.14 (MN-2022)</t>
+          <t>9.2.4.1 (MN-2022), 9.2.4.12 (MN-2022), 9.2.4.13 (MN-2022), 9.2.4.14 (MN-2022), 7.NS.A.1.A (CCSS-M), 7.SP.7a (CCSS-M), 7.SP.7b (CCSS-M), 7.SP.7c (CCSS-M)</t>
         </is>
       </c>
     </row>
@@ -52127,11 +52327,11 @@
         </is>
       </c>
       <c r="G499" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="H499" s="8" t="inlineStr">
         <is>
-          <t>9.2.4.1 (MN-2022), 9.2.4.7 (MN-2022), 9.2.4.12 (MN-2022)</t>
+          <t>9.2.4.1 (MN-2022), 9.2.4.7 (MN-2022), 9.2.4.12 (MN-2022), 7.NS.A.1.A (CCSS-M), 7.RP.A.2.B (CCSS-M), 7.SP.7a (CCSS-M)</t>
         </is>
       </c>
     </row>
@@ -52157,11 +52357,11 @@
         </is>
       </c>
       <c r="G500" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H500" s="8" t="inlineStr">
         <is>
-          <t>9.2.3.6 (MN-2022), 9.2.4.12 (MN-2022)</t>
+          <t>9.2.3.6 (MN-2022), 9.2.4.12 (MN-2022), 5.NF.A.1 (CCSS-M), 7.SP.7a (CCSS-M)</t>
         </is>
       </c>
     </row>
@@ -52187,11 +52387,11 @@
         </is>
       </c>
       <c r="G501" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H501" s="8" t="inlineStr">
         <is>
-          <t>9.2.3.9 (MN-2022)</t>
+          <t>9.2.3.9 (MN-2022), 7.NS.A.1.D (CCSS-M)</t>
         </is>
       </c>
     </row>
@@ -52217,11 +52417,11 @@
         </is>
       </c>
       <c r="G502" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="H502" s="8" t="inlineStr">
         <is>
-          <t>9.2.3.3 (MN-2022), 9.2.3.8 (MN-2022), 9.2.4.12 (MN-2022)</t>
+          <t>9.2.3.3 (MN-2022), 9.2.3.8 (MN-2022), 9.2.4.12 (MN-2022), 7.SP.C.7.B (CCSS-M), 7.SP.C.8.A (CCSS-M), 7.SP.7a (CCSS-M)</t>
         </is>
       </c>
     </row>
@@ -52243,11 +52443,11 @@
       <c r="E503" s="7" t="n"/>
       <c r="F503" s="8" t="inlineStr"/>
       <c r="G503" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H503" s="8" t="inlineStr">
         <is>
-          <t>9.2.3.3 (MN-2022), 9.2.3.8 (MN-2022)</t>
+          <t>9.2.3.3 (MN-2022), 9.2.3.8 (MN-2022), 7.SP.C.7.B (CCSS-M), 7.SP.C.8.A (CCSS-M)</t>
         </is>
       </c>
     </row>
@@ -52269,11 +52469,11 @@
       <c r="E504" s="7" t="n"/>
       <c r="F504" s="8" t="inlineStr"/>
       <c r="G504" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="H504" s="8" t="inlineStr">
         <is>
-          <t>9.1.2.8 (MN-2022), 9.2.3.2 (MN-2022), 9.2.3.3 (MN-2022)</t>
+          <t>9.1.2.8 (MN-2022), 9.2.3.2 (MN-2022), 9.2.3.3 (MN-2022), 7.SP.C.8.C (CCSS-M), 7.NS.A.2.D (CCSS-M), 7.SP.C.7.B (CCSS-M)</t>
         </is>
       </c>
     </row>
@@ -52295,11 +52495,11 @@
       <c r="E505" s="7" t="n"/>
       <c r="F505" s="8" t="inlineStr"/>
       <c r="G505" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H505" s="8" t="inlineStr">
         <is>
-          <t>9.2.3.2 (MN-2022), 9.2.3.3 (MN-2022)</t>
+          <t>9.2.3.2 (MN-2022), 9.2.3.3 (MN-2022), 7.NS.A.2.D (CCSS-M), 7.SP.C.7.B (CCSS-M)</t>
         </is>
       </c>
     </row>
@@ -52321,11 +52521,11 @@
       <c r="E506" s="7" t="n"/>
       <c r="F506" s="8" t="inlineStr"/>
       <c r="G506" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="H506" s="8" t="inlineStr">
         <is>
-          <t>9.2.4.4 (MN-2022), 9.2.4.5 (MN-2022), 9.2.4.7 (MN-2022), 9.2.4.10 (MN-2022)</t>
+          <t>9.2.4.4 (MN-2022), 9.2.4.5 (MN-2022), 9.2.4.7 (MN-2022), 9.2.4.10 (MN-2022), 7.NS.A.2.C (CCSS-M), 7.RP.A.2.A (CCSS-M), 7.RP.A.2.B (CCSS-M), 7.RP.3 (CCSS-M)</t>
         </is>
       </c>
     </row>
@@ -52347,11 +52547,11 @@
       <c r="E507" s="7" t="n"/>
       <c r="F507" s="8" t="inlineStr"/>
       <c r="G507" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H507" s="8" t="inlineStr">
         <is>
-          <t>9.2.3.1 (MN-2022), 9.2.4.10 (MN-2022)</t>
+          <t>9.2.3.1 (MN-2022), 9.2.4.10 (MN-2022), 8.EE.C.7.B (CCSS-M), 7.RP.3 (CCSS-M)</t>
         </is>
       </c>
     </row>
@@ -52377,11 +52577,11 @@
         </is>
       </c>
       <c r="G508" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="H508" s="8" t="inlineStr">
         <is>
-          <t>9.1.2.1 (MN-2022), 9.1.2.2 (MN-2022), 9.1.2.3 (MN-2022), 9.1.2.4 (MN-2022), 9.1.2.7 (MN-2022)</t>
+          <t>9.1.2.1 (MN-2022), 9.1.2.2 (MN-2022), 9.1.2.3 (MN-2022), 9.1.2.4 (MN-2022), 9.1.2.7 (MN-2022), 6.EE.A.4 (CCSS-M), 6.EE.A.2.C (CCSS-M), Review skills needed for 6.NS.1 (CCSS-M), 6.RP.3c (CCSS-M), 6.G.1 (CCSS-M)</t>
         </is>
       </c>
     </row>
@@ -52403,11 +52603,11 @@
       <c r="E509" s="7" t="n"/>
       <c r="F509" s="8" t="inlineStr"/>
       <c r="G509" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H509" s="8" t="inlineStr">
         <is>
-          <t>9.2.4.15 (MN-2022)</t>
+          <t>9.2.4.15 (MN-2022), 7.SP.6 (CCSS-M)</t>
         </is>
       </c>
     </row>
@@ -52429,11 +52629,11 @@
       <c r="E510" s="7" t="n"/>
       <c r="F510" s="8" t="inlineStr"/>
       <c r="G510" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="H510" s="8" t="inlineStr">
         <is>
-          <t>9.2.4.3 (MN-2022), 9.2.4.4 (MN-2022), 9.2.4.7 (MN-2022)</t>
+          <t>9.2.4.3 (MN-2022), 9.2.4.4 (MN-2022), 9.2.4.7 (MN-2022), 7.NS.A.2.A (CCSS-M), 7.NS.A.2.C (CCSS-M), 7.RP.A.2.B (CCSS-M)</t>
         </is>
       </c>
     </row>
@@ -52455,11 +52655,11 @@
       <c r="E511" s="7" t="n"/>
       <c r="F511" s="8" t="inlineStr"/>
       <c r="G511" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H511" s="8" t="inlineStr">
         <is>
-          <t>9.2.3.1 (MN-2022)</t>
+          <t>9.2.3.1 (MN-2022), 8.EE.C.7.B (CCSS-M)</t>
         </is>
       </c>
     </row>
@@ -52511,11 +52711,11 @@
         </is>
       </c>
       <c r="G513" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="H513" s="8" t="inlineStr">
         <is>
-          <t>9.2.4.4 (MN-2022), 9.2.4.6 (MN-2022), 9.2.4.7 (MN-2022), 9.2.4.10 (MN-2022), 9.2.4.11 (MN-2022), 9.2.4.12 (MN-2022)</t>
+          <t>9.2.4.4 (MN-2022), 9.2.4.6 (MN-2022), 9.2.4.7 (MN-2022), 9.2.4.10 (MN-2022), 9.2.4.11 (MN-2022), 9.2.4.12 (MN-2022), 7.NS.A.2.C (CCSS-M), 7.RP.A.2.D (CCSS-M), 7.RP.A.2.B (CCSS-M), 7.RP.3 (CCSS-M) +1 more</t>
         </is>
       </c>
     </row>
@@ -52537,11 +52737,11 @@
       <c r="E514" s="7" t="n"/>
       <c r="F514" s="8" t="inlineStr"/>
       <c r="G514" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="H514" s="8" t="inlineStr">
         <is>
-          <t>9.2.3.3 (MN-2022), 9.2.4.1 (MN-2022), 9.2.4.3 (MN-2022), 9.2.4.12 (MN-2022), 9.2.4.15 (MN-2022)</t>
+          <t>9.2.3.3 (MN-2022), 9.2.4.1 (MN-2022), 9.2.4.3 (MN-2022), 9.2.4.12 (MN-2022), 9.2.4.15 (MN-2022), 7.SP.C.7.B (CCSS-M), 7.NS.A.1.A (CCSS-M), 7.NS.A.2.A (CCSS-M), 7.SP.7a (CCSS-M), 7.SP.6 (CCSS-M)</t>
         </is>
       </c>
     </row>
@@ -52563,11 +52763,11 @@
       <c r="E515" s="7" t="n"/>
       <c r="F515" s="8" t="inlineStr"/>
       <c r="G515" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H515" s="8" t="inlineStr">
         <is>
-          <t>9.2.3.9 (MN-2022)</t>
+          <t>9.2.3.9 (MN-2022), 7.NS.A.1.D (CCSS-M)</t>
         </is>
       </c>
     </row>
@@ -52589,11 +52789,11 @@
       <c r="E516" s="7" t="n"/>
       <c r="F516" s="8" t="inlineStr"/>
       <c r="G516" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H516" s="8" t="inlineStr">
         <is>
-          <t>9.2.4.3 (MN-2022)</t>
+          <t>9.2.4.3 (MN-2022), 7.NS.A.2.A (CCSS-M)</t>
         </is>
       </c>
     </row>
@@ -52619,11 +52819,11 @@
         </is>
       </c>
       <c r="G517" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H517" s="8" t="inlineStr">
         <is>
-          <t>9.2.3.3 (MN-2022), 9.2.4.12 (MN-2022)</t>
+          <t>9.2.3.3 (MN-2022), 9.2.4.12 (MN-2022), 7.SP.C.7.B (CCSS-M), 7.SP.7a (CCSS-M)</t>
         </is>
       </c>
     </row>
@@ -52645,11 +52845,11 @@
       <c r="E518" s="7" t="n"/>
       <c r="F518" s="8" t="inlineStr"/>
       <c r="G518" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H518" s="8" t="inlineStr">
         <is>
-          <t>9.2.3.4 (MN-2022), 9.2.3.9 (MN-2022)</t>
+          <t>9.2.3.4 (MN-2022), 9.2.3.9 (MN-2022), 7.SP.C.7.A (CCSS-M), 7.NS.A.1.D (CCSS-M)</t>
         </is>
       </c>
     </row>
@@ -52671,11 +52871,11 @@
       <c r="E519" s="7" t="n"/>
       <c r="F519" s="8" t="inlineStr"/>
       <c r="G519" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H519" s="8" t="inlineStr">
         <is>
-          <t>9.2.4.1 (MN-2022), 9.2.4.12 (MN-2022)</t>
+          <t>9.2.4.1 (MN-2022), 9.2.4.12 (MN-2022), 7.NS.A.1.A (CCSS-M), 7.SP.7a (CCSS-M)</t>
         </is>
       </c>
     </row>
@@ -52697,11 +52897,11 @@
       <c r="E520" s="7" t="n"/>
       <c r="F520" s="8" t="inlineStr"/>
       <c r="G520" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H520" s="8" t="inlineStr">
         <is>
-          <t>9.2.4.8 (MN-2022), 9.2.4.9 (MN-2022)</t>
+          <t>9.2.4.8 (MN-2022), 9.2.4.9 (MN-2022), 7.NS.A.1.C (CCSS-M), 7.RP.A.2.C (CCSS-M)</t>
         </is>
       </c>
     </row>
@@ -52723,11 +52923,11 @@
       <c r="E521" s="7" t="n"/>
       <c r="F521" s="8" t="inlineStr"/>
       <c r="G521" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="H521" s="8" t="inlineStr">
         <is>
-          <t>9.1.2.1 (MN-2022), 9.1.2.3 (MN-2022), 9.1.2.5 (MN-2022)</t>
+          <t>9.1.2.1 (MN-2022), 9.1.2.3 (MN-2022), 9.1.2.5 (MN-2022), 6.EE.A.4 (CCSS-M), Review skills needed for 6.NS.1 (CCSS-M), 6.NS.3 (CCSS-M)</t>
         </is>
       </c>
     </row>
@@ -52749,11 +52949,11 @@
       <c r="E522" s="7" t="n"/>
       <c r="F522" s="8" t="inlineStr"/>
       <c r="G522" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H522" s="8" t="inlineStr">
         <is>
-          <t>9.1.2.1 (MN-2022)</t>
+          <t>9.1.2.1 (MN-2022), 6.EE.A.4 (CCSS-M)</t>
         </is>
       </c>
     </row>
@@ -52775,11 +52975,11 @@
       <c r="E523" s="7" t="n"/>
       <c r="F523" s="8" t="inlineStr"/>
       <c r="G523" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H523" s="8" t="inlineStr">
         <is>
-          <t>9.2.3.4 (MN-2022), 9.2.3.5 (MN-2022)</t>
+          <t>9.2.3.4 (MN-2022), 9.2.3.5 (MN-2022), 7.SP.C.7.A (CCSS-M), Prep for 7.SP.C.8.A (CCSS-M)</t>
         </is>
       </c>
     </row>
@@ -52801,11 +53001,11 @@
       <c r="E524" s="7" t="n"/>
       <c r="F524" s="8" t="inlineStr"/>
       <c r="G524" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="H524" s="8" t="inlineStr">
         <is>
-          <t>9.2.3.5 (MN-2022), 9.2.4.8 (MN-2022), 9.2.4.9 (MN-2022), 9.2.4.12 (MN-2022)</t>
+          <t>9.2.3.5 (MN-2022), 9.2.4.8 (MN-2022), 9.2.4.9 (MN-2022), 9.2.4.12 (MN-2022), Prep for 7.SP.C.8.A (CCSS-M), 7.NS.A.1.C (CCSS-M), 7.RP.A.2.C (CCSS-M), 7.SP.7a (CCSS-M)</t>
         </is>
       </c>
     </row>
@@ -52827,11 +53027,11 @@
       <c r="E525" s="7" t="n"/>
       <c r="F525" s="8" t="inlineStr"/>
       <c r="G525" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="H525" s="8" t="inlineStr">
         <is>
-          <t>9.2.3.3 (MN-2022), 9.2.4.12 (MN-2022), 9.3.6.6 (MN-2022)</t>
+          <t>9.2.3.3 (MN-2022), 9.2.4.12 (MN-2022), 9.3.6.6 (MN-2022), 7.SP.C.7.B (CCSS-M), 7.SP.7a (CCSS-M), MP4 (CCSS-M)</t>
         </is>
       </c>
     </row>
@@ -72393,7 +72593,7 @@
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="50" customWidth="1" min="2" max="2"/>
     <col width="50" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
     <col width="50" customWidth="1" min="5" max="5"/>
     <col width="50" customWidth="1" min="6" max="6"/>
   </cols>
@@ -72453,7 +72653,11 @@
           <t>9.3.6.7, 9.3.7.1, 9.3.7.2, 9.3.7.7</t>
         </is>
       </c>
-      <c r="D3" s="16" t="inlineStr"/>
+      <c r="D3" s="16" t="inlineStr">
+        <is>
+          <t>7.EE.A.1.A, 8.EE.A.8, 8.EE.C.7.A</t>
+        </is>
+      </c>
       <c r="E3" s="17" t="inlineStr">
         <is>
           <t>TF: 1-1 to 3, 9 to 12; Team: 1-23, (24)</t>
@@ -72489,7 +72693,11 @@
           <t>9.3.7.1, 9.3.7.2, 9.3.7.7</t>
         </is>
       </c>
-      <c r="D5" s="16" t="inlineStr"/>
+      <c r="D5" s="16" t="inlineStr">
+        <is>
+          <t>7.EE.A.1.A, 8.EE.A.8, 8.EE.C.7.A</t>
+        </is>
+      </c>
       <c r="E5" s="17" t="inlineStr">
         <is>
           <t>TF: 2-25, 36-37; Team: 2-14 to 16, (17-18), 25-27, 38-39; IS: 2-11 to 13, (28-29), 30 (LL), 40 (LL)</t>
@@ -72518,7 +72726,11 @@
           <t>9.2.3.6, 9.3.7.1, 9.3.7.7</t>
         </is>
       </c>
-      <c r="D6" s="16" t="inlineStr"/>
+      <c r="D6" s="16" t="inlineStr">
+        <is>
+          <t>5.NF.A.1, 8.EE.A.8, 8.EE.C.7.A</t>
+        </is>
+      </c>
       <c r="E6" s="17" t="inlineStr">
         <is>
           <t>TF: 2-(46, 47), 53; Team: 2-54 to 57, 68; IS: 2-58 (LL), 69</t>
@@ -72578,7 +72790,11 @@
           <t>9.3.5.8, 9.3.6.1, 9.3.7.1</t>
         </is>
       </c>
-      <c r="D9" s="16" t="inlineStr"/>
+      <c r="D9" s="16" t="inlineStr">
+        <is>
+          <t>7.EE.3, 7.SP.8a, 8.EE.C.7.A</t>
+        </is>
+      </c>
       <c r="E9" s="17" t="inlineStr">
         <is>
           <t>TF: (3-25 to 32 as needed), 3-45, 56, 65 to 67; Team: 3-46, (54), 55, 68, (69); IS: 3-47 (LL), 57, 6</t>
@@ -72613,7 +72829,11 @@
           <t>9.3.7.1</t>
         </is>
       </c>
-      <c r="D11" s="16" t="inlineStr"/>
+      <c r="D11" s="16" t="inlineStr">
+        <is>
+          <t>8.EE.C.7.A</t>
+        </is>
+      </c>
       <c r="E11" s="17" t="inlineStr">
         <is>
           <t>TF: 4-20 to 23; Team: 4-1 to 3, (4-5), 6, (7), (24)</t>
@@ -72642,7 +72862,11 @@
           <t>9.3.7.1</t>
         </is>
       </c>
-      <c r="D12" s="16" t="inlineStr"/>
+      <c r="D12" s="16" t="inlineStr">
+        <is>
+          <t>8.EE.C.7.A</t>
+        </is>
+      </c>
       <c r="E12" s="17" t="inlineStr">
         <is>
           <t>TF: 4-32 to 34, (35-41), 42, 55-56; Team: 4-33 to 34, (35), 43-45, 57-59, 67-70, 77-79; IS: 4-31, (4</t>
@@ -72678,7 +72902,11 @@
           <t>9.3.7.1, 9.3.7.4, 9.3.7.5</t>
         </is>
       </c>
-      <c r="D14" s="16" t="inlineStr"/>
+      <c r="D14" s="16" t="inlineStr">
+        <is>
+          <t>7.EE.B.4.B, 8.EE.B.8, 8.EE.C.7.A</t>
+        </is>
+      </c>
       <c r="E14" s="17" t="inlineStr">
         <is>
           <t>TF: 2020-05-01 00:00:00; Team: 2020-05-03 00:00:00; IS: 5-4 and 5-5 LL
@@ -72707,7 +72935,11 @@
           <t>9.3.7.4, 9.3.7.5</t>
         </is>
       </c>
-      <c r="D15" s="16" t="inlineStr"/>
+      <c r="D15" s="16" t="inlineStr">
+        <is>
+          <t>7.EE.B.4.B, 8.EE.B.8</t>
+        </is>
+      </c>
       <c r="E15" s="17" t="inlineStr">
         <is>
           <t>TF: 5-40; Team: 5-41 
@@ -72736,7 +72968,11 @@
           <t>9.3.5.5, 9.3.7.1, 9.3.7.4, 9.3.7.5, 9.3.7.7</t>
         </is>
       </c>
-      <c r="D16" s="16" t="inlineStr"/>
+      <c r="D16" s="16" t="inlineStr">
+        <is>
+          <t>7.EE.B.4.B, 8.EE.A.8, 8.EE.B.8, 8.EE.C.7.A</t>
+        </is>
+      </c>
       <c r="E16" s="17" t="inlineStr">
         <is>
           <t>Team: 5-82 (eTool), 5-83 (eTool), 5-84</t>
@@ -72771,7 +73007,11 @@
           <t>9.1.1.11, 9.1.1.6, 9.2.3.6, 9.3.5.6, 9.3.7.1</t>
         </is>
       </c>
-      <c r="D18" s="16" t="inlineStr"/>
+      <c r="D18" s="16" t="inlineStr">
+        <is>
+          <t>5.NF.A.1, 6.RP.A.3.C, 7.Sp.8a, 8.EE.C.7.A</t>
+        </is>
+      </c>
       <c r="E18" s="17" t="inlineStr">
         <is>
           <t>TF: 6-1a; Team: 6-1 b-d, 6-2; IS: 2020-06-03 00:00:00</t>
@@ -72799,7 +73039,11 @@
           <t>9.1.1.11, 9.1.1.15, 9.1.1.5, 9.1.1.6, 9.1.1.8, 9.2.3.6, 9.3.5.6</t>
         </is>
       </c>
-      <c r="D19" s="16" t="inlineStr"/>
+      <c r="D19" s="16" t="inlineStr">
+        <is>
+          <t>5.NF.A.1, 6.EE.A.2.A, 6.EE.A.3, 6.NS.C.6.B, 6.RP.A.3.C, 7.Sp.8a</t>
+        </is>
+      </c>
       <c r="E19" s="17" t="inlineStr">
         <is>
           <t>TF: 6-48; Team: 6-49, 6-50; IS: 6-51, LL 6-54</t>
@@ -72834,7 +73078,11 @@
           <t>9.3.7.10, 9.3.7.2, 9.3.7.3, 9.3.7.6, 9.3.7.7</t>
         </is>
       </c>
-      <c r="D21" s="16" t="inlineStr"/>
+      <c r="D21" s="16" t="inlineStr">
+        <is>
+          <t>7.EE.A.1.A, 7.EE.A.1.B, 8.EE.A.8, 8.EE.B.7, 8.G.2</t>
+        </is>
+      </c>
       <c r="E21" s="17" t="inlineStr">
         <is>
           <t>TF: 1-30, 31; Team: 1-(43 to 45), 63-64, 71-77; IS: 1-32 (LL), (46), 52-55, (56), 62, 65 (LL)</t>
@@ -72862,7 +73110,11 @@
           <t>9.2.3.6, 9.3.5.6, 9.3.7.1</t>
         </is>
       </c>
-      <c r="D22" s="16" t="inlineStr"/>
+      <c r="D22" s="16" t="inlineStr">
+        <is>
+          <t>5.NF.A.1, 7.Sp.8a, 8.EE.C.7.A</t>
+        </is>
+      </c>
       <c r="E22" s="17" t="inlineStr">
         <is>
           <t>Team: Select from 4-87 to 97</t>
@@ -72890,7 +73142,11 @@
           <t>9.2.3.6, 9.3.7.1, 9.3.7.2, 9.3.7.6, 9.3.7.7, 9.3.7.8</t>
         </is>
       </c>
-      <c r="D23" s="16" t="inlineStr"/>
+      <c r="D23" s="16" t="inlineStr">
+        <is>
+          <t>5.NF.A.1, 7.EE.A.1.A, 8.EE.A.8, 8.EE.B.7, 8.EE.C.7.A, 8.G.B.1</t>
+        </is>
+      </c>
       <c r="E23" s="17" t="inlineStr">
         <is>
           <t>TF: 2020-07-01 00:00:00; Team: 7-2, 7-3; IS: 7-5, LL 7-6</t>
@@ -72918,7 +73174,11 @@
           <t>9.3.5.2, 9.3.5.6, 9.3.6.8, 9.3.7.1, 9.3.7.2</t>
         </is>
       </c>
-      <c r="D24" s="16" t="inlineStr"/>
+      <c r="D24" s="16" t="inlineStr">
+        <is>
+          <t>7.EE.A.1.A, 7.Sp.8a, 8.EE.C.7.A, MP8</t>
+        </is>
+      </c>
       <c r="E24" s="17" t="inlineStr">
         <is>
           <t>TF: 7-79, 7-80; Team: 7-81, 7-82, 7-83; IS: LL 7-86</t>
@@ -72953,7 +73213,11 @@
           <t>9.2.3.6, 9.3.7.1</t>
         </is>
       </c>
-      <c r="D26" s="16" t="inlineStr"/>
+      <c r="D26" s="16" t="inlineStr">
+        <is>
+          <t>5.NF.A.1, 8.EE.C.7.A</t>
+        </is>
+      </c>
       <c r="E26" s="17" t="inlineStr">
         <is>
           <t>TF: 2-75 to 78; Team: 2-79, (80), (87-88); IS: 2-81 (LL), 89 (LL), 95 (Desmos)</t>
@@ -72982,7 +73246,11 @@
           <t>9.3.5.7, 9.3.5.8, 9.3.6.2, 9.3.6.4</t>
         </is>
       </c>
-      <c r="D27" s="16" t="inlineStr"/>
+      <c r="D27" s="16" t="inlineStr">
+        <is>
+          <t>7.EE.4b, 7.SP.8a</t>
+        </is>
+      </c>
       <c r="E27" s="17" t="inlineStr">
         <is>
           <t>TF: 8-1, 8-2 a; Team: 8-2 b &amp; c, 8-3 a &amp; b, 8-4; IS: LL 8-5</t>
@@ -73010,7 +73278,11 @@
           <t>9.2.3.6, 9.3.5.7, 9.3.5.8, 9.3.6.2, 9.3.6.3, 9.3.6.5, 9.3.7.1, 9.3.7.2, 9.3.7.7</t>
         </is>
       </c>
-      <c r="D28" s="16" t="inlineStr"/>
+      <c r="D28" s="16" t="inlineStr">
+        <is>
+          <t>5.NF.A.1, 7.EE.4a, 7.EE.A.1.A, 7.SP.8a, 8.EE.A.8, 8.EE.C.7.A, see ebook</t>
+        </is>
+      </c>
       <c r="E28" s="17" t="inlineStr">
         <is>
           <t>TF: 8-56; Team: 8-55; IS: LL 8-57</t>
@@ -73045,7 +73317,11 @@
           <t>9.3.6.3, 9.3.6.5</t>
         </is>
       </c>
-      <c r="D30" s="16" t="inlineStr"/>
+      <c r="D30" s="16" t="inlineStr">
+        <is>
+          <t>7.EE.4a, see ebook</t>
+        </is>
+      </c>
       <c r="E30" s="17" t="inlineStr">
         <is>
           <t>TF: 9-3, 9-4a; Team: 9-1, 9-2, 9-4b</t>
@@ -73073,7 +73349,11 @@
           <t>9.3.7.1</t>
         </is>
       </c>
-      <c r="D31" s="16" t="inlineStr"/>
+      <c r="D31" s="16" t="inlineStr">
+        <is>
+          <t>8.EE.C.7.A</t>
+        </is>
+      </c>
       <c r="E31" s="17" t="inlineStr">
         <is>
           <t>TF: 9-44, 9-45; Team: 9-46, 9-47, 9-48; IS: 9-49</t>
@@ -73125,7 +73405,11 @@
           <t>9.3.7.1</t>
         </is>
       </c>
-      <c r="D33" s="16" t="inlineStr"/>
+      <c r="D33" s="16" t="inlineStr">
+        <is>
+          <t>8.EE.C.7.A</t>
+        </is>
+      </c>
       <c r="E33" s="17" t="inlineStr">
         <is>
           <t>TF: 9-89, 9-91; Team: 9-90, 9-92</t>
@@ -73160,7 +73444,11 @@
           <t>9.1.2.5</t>
         </is>
       </c>
-      <c r="D35" s="16" t="inlineStr"/>
+      <c r="D35" s="16" t="inlineStr">
+        <is>
+          <t>6.NS.3</t>
+        </is>
+      </c>
       <c r="E35" s="17" t="inlineStr">
         <is>
           <t>TF: 10-1, 10-2; Team: 10-3, 10-4</t>
@@ -73188,7 +73476,11 @@
           <t>9.3.5.3, 9.3.5.7, 9.3.5.8</t>
         </is>
       </c>
-      <c r="D36" s="16" t="inlineStr"/>
+      <c r="D36" s="16" t="inlineStr">
+        <is>
+          <t>7.SP.8a, 7.SP.8b</t>
+        </is>
+      </c>
       <c r="E36" s="17" t="inlineStr">
         <is>
           <t>TF: 10-22, 10-24; Team: 10-23, 10-25</t>
@@ -73240,7 +73532,11 @@
           <t>9.3.5.7, 9.3.5.8</t>
         </is>
       </c>
-      <c r="D38" s="16" t="inlineStr"/>
+      <c r="D38" s="16" t="inlineStr">
+        <is>
+          <t>7.SP.8a</t>
+        </is>
+      </c>
       <c r="E38" s="17" t="inlineStr">
         <is>
           <t>TF: 3-78 to 79, 87-89; Team: 3-77,80,90-91,105; IS: 3-(76), (92), 106 (LL)</t>
@@ -73277,7 +73573,11 @@
           <t>9.3.7.2, 9.3.7.3, 9.3.7.9</t>
         </is>
       </c>
-      <c r="D40" s="16" t="inlineStr"/>
+      <c r="D40" s="16" t="inlineStr">
+        <is>
+          <t>7.EE.A.1.A, 7.EE.A.1.B, 8.G.C.1</t>
+        </is>
+      </c>
       <c r="E40" s="17" t="inlineStr">
         <is>
           <t>TF: 2021-11-01 00:00:00; Team: 2021-11-02 00:00:00; IS: LL 11-3</t>
@@ -73305,7 +73605,11 @@
           <t>9.1.1.10, 9.1.1.13, 9.1.1.7, 9.1.1.9</t>
         </is>
       </c>
-      <c r="D41" s="16" t="inlineStr"/>
+      <c r="D41" s="16" t="inlineStr">
+        <is>
+          <t>6.NS.C.6.A, 6.NS.C.7.A, 6.NS.C.7.B, 6.NS.C.7.D</t>
+        </is>
+      </c>
       <c r="E41" s="17" t="inlineStr">
         <is>
           <t>Team: 2021-11-26 00:00:00; IS: LL 11-27</t>
@@ -73333,7 +73637,11 @@
           <t>9.2.3.7, 9.3.7.1</t>
         </is>
       </c>
-      <c r="D42" s="16" t="inlineStr"/>
+      <c r="D42" s="16" t="inlineStr">
+        <is>
+          <t>8.EE.C.7.A</t>
+        </is>
+      </c>
       <c r="E42" s="17" t="inlineStr"/>
       <c r="F42" s="17" t="inlineStr">
         <is>

</xml_diff>